<commit_message>
Run pipeline metrics against sample data
</commit_message>
<xml_diff>
--- a/data/sample/sample_personal_statements.xlsx
+++ b/data/sample/sample_personal_statements.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,444 +413,767 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>ApplicantNumber</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>YearOfEntry</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>StatementText</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>applicationCourse</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>applicationCourse_titlemain</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>subject</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>personal_statement</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>I am applying for a degree in Accounting as I believe this degree will set me in good stead for my future career. In recent years I have become interested in the world of commerce and industry and I believe that studying this subject at university level will help me reach my goal of becoming an accountant. I have researched this career and believe that I have the necessary skills to succeed. At my college, all year 12 students undertake a week’s work experience in July. I arranged for mine to be at Phillips and Woodstock, a small accountancy firm in my local town. During this week I learned that there are several elements of the accountancy profession and that the career is very diverse. Phillips and Woodstock specialise in helping small businesses with their tax assessments, and as a result I have become particularly interested in the business consultancy side of accounting. The MD, Mr Phillips, was impressed with my work and commitment and has invited me to work at the firm part-time in my summer holidays. I am looking forward to the opportunity to gain more experience in my chosen career. I am currently studying towards a BTEC Level 3 Extended Diploma in Business. The modules I have most enjoyed are ‘Managing Information’ and ‘Managing a Business Project or an Event’. For the latter module my project was based on a tender by a construction company where I took the role of estimator and tried to write a competitive tender proposal. This was a challenging and interesting task, and one which taught me the importance of expertise in a chosen field. However it was the unit ‘Introduction to Accounting’ which I most enjoyed and which, in retrospect, first sparked my interest in accounting. I have a part-time job in a roadside restaurant near to my home. Although the job can be repetitive, it has been an important exercise in self-discipline as I start work at 7am on Saturdays! I have also met many new people and become friends with some of the regulars. I try to save the money I earn from this job: university has been my long-term goal for the last year and my savings should help with the costs of studying. I am really looking forward to going to university: partly for the social experience, but most importantly to further my studies in accounting. I believe that university will help me achieve my aim of qualifying as an accountant and perhaps one day running my own business, like Mr Phillips, or my all-time hero, Sir Alan Sugar. I would hope, however, never to be fired!</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>BSC X924 ACCOUNTING, FINANCE AND BANKING</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ACCOUNTING, FINANCE AND BANKING</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
         <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ACCOUNTING, FINANCE AND BANKING</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>I am applying for a degree in Accounting as I believe this degree will set me in good stead for my future career. In recent years I have become interested in the world of commerce and industry and I believe that studying this subject at university level will help me reach my goal of becoming an accountant. I have researched this career and believe that I have the necessary skills to succeed. At my college, all year 12 students undertake a week’s work experience in July. I arranged for mine to be at Phillips and Woodstock, a small accountancy firm in my local town. During this week I learned that there are several elements of the accountancy profession and that the career is very diverse. Phillips and Woodstock specialise in helping small businesses with their tax assessments, and as a result I have become particularly interested in the business consultancy side of accounting. The MD, Mr Phillips, was impressed with my work and commitment and has invited me to work at the firm part-time in my summer holidays. I am looking forward to the opportunity to gain more experience in my chosen career. I am currently studying towards a BTEC Level 3 Extended Diploma in Business. The modules I have most enjoyed are ‘Managing Information’ and ‘Managing a Business Project or an Event’. For the latter module my project was based on a tender by a construction company where I took the role of estimator and tried to write a competitive tender proposal. This was a challenging and interesting task, and one which taught me the importance of expertise in a chosen field. However it was the unit ‘Introduction to Accounting’ which I most enjoyed and which, in retrospect, first sparked my interest in accounting. I have a part-time job in a roadside restaurant near to my home. Although the job can be repetitive, it has been an important exercise in self-discipline as I start work at 7am on Saturdays! I have also met many new people and become friends with some of the regulars. I try to save the money I earn from this job: university has been my long-term goal for the last year and my savings should help with the costs of studying. I am really looking forward to going to university: partly for the social experience, but most importantly to further my studies in accounting. I believe that university will help me achieve my aim of qualifying as an accountant and perhaps one day running my own business, like Mr Phillips, or my all-time hero, Sir Alan Sugar. I would hope, however, never to be fired!</t>
-        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
+        <v>1001</v>
+      </c>
+      <c r="B3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>‘Nature has established patterns originating in the return of events, but only for the most part’. It is the latter part of Gottfried von Leibniz’s comment in 1703 that lays the foundations of the existence of risk. Without risk, we would live in a dull world where all future events are predictable, and no change ever occurred. It is the ability to quantify risk that enables secure financial growth, both personal and professional, as well as the power to foresee any financial disasters that may be prevented. For this, we rely on the work of Actuaries, a career that I am determined will become my future. In my free time I decided to turn my attention to Bernstein’s Against the Gods: The Remarkable Story of Risk, which gave me an insight into the history and development of the notion of risk. However, it was the deterministic chaos theory that really interested me after reading James Gleik’s Chaos: The Amazing Science of the Unpredictable, an active example of actuarial modelling, where the most miniscule changes in the initial conditions have the ability to cause substantial disasters in the future. My obsession with maths was pronounced right from secondary school. I completed my GCSE Mathematics in November 2010, gaining a solid A*, before moving on to studying the edexcel Free Standing Maths Qualification; Additional Maths. In year 10, I also took part in the West Midlands Maths Challenge after being placed second in the Birmingham Maths Challenge, and used my free time to write a 1500 Word essay titled ‘Should Zero Be considered a Number?’ However, it is the statistics and probability area that my fascination heavily lies, evident in my result of 96 UMS points in the AQA Statistics exam. It is, primarily, the most important application of mathematical concepts to real-life situations. In particular, I enjoy carrying out Chi-square tests to determine any association between two variables. This is because of its complicated process, and the need to identify the necessary use of Yates’ correction, or the grouping of data too small, to obtain accurate results. I find a great sense of achievement on completion of these tests, as well as many other processes studied in statistics. The fact that a large part of Actuarial Science involves analysing statistical data, needed to assess the future effects of large financial risks, is what draws me to the degree. I understand the Actuary profession is not an easy one, but one that requires dedication and motivation, something I have proven to be great qualities of mine. Since the age of 15, I have had at least one job at any time, holding two part-time jobs whilst taking my A-levels; with my results proving my handling of this to have been successful. As a part-time receptionist for three years, from the age of 15, I have developed strong communication and interpersonal skills. This will enable me to effectively convey my knowledge of complex financial information to non-specialists, essential for someone entering the Actuarial profession. My attraction to the degree, as well as my suitability to the career is clear. It is my desire to learn and my constant search for a challenge that draws me to this path. I thrive on spontaneity, and knowing of the diverse and wide-ranging activities an Actuary can find themselves responsible for in their day-to-day work, from analysing risk and calculating profit, to developing and overseeing new financial products, I find myself impatient to start my studies in Actuarial Science. In the meantime, I plan to spend the year keeping up to date with current world financial affairs and to take work experience where possible, so that I am thoroughly prepared to begin a successful Actuarial career path in 2014. 13 Did you know...  The starting salary of actuarial graduates is on average upwards of £30,000.  Our course is accredited by the Institute and Faculty of Actuaries for the purpose of exemption from some professional examinations.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>BSC V304 ACTUARIAL SCIENCE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ACTUARIAL SCIENCE</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ACTUARIAL SCIENCE</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>‘Nature has established patterns originating in the return of events, but only for the most part’. It is the latter part of Gottfried von Leibniz’s comment in 1703 that lays the foundations of the existence of risk. Without risk, we would live in a dull world where all future events are predictable, and no change ever occurred. It is the ability to quantify risk that enables secure financial growth, both personal and professional, as well as the power to foresee any financial disasters that may be prevented. For this, we rely on the work of Actuaries, a career that I am determined will become my future. In my free time I decided to turn my attention to Bernstein’s Against the Gods: The Remarkable Story of Risk, which gave me an insight into the history and development of the notion of risk. However, it was the deterministic chaos theory that really interested me after reading James Gleik’s Chaos: The Amazing Science of the Unpredictable, an active example of actuarial modelling, where the most miniscule changes in the initial conditions have the ability to cause substantial disasters in the future. My obsession with maths was pronounced right from secondary school. I completed my GCSE Mathematics in November 2010, gaining a solid A*, before moving on to studying the edexcel Free Standing Maths Qualification; Additional Maths. In year 10, I also took part in the West Midlands Maths Challenge after being placed second in the Birmingham Maths Challenge, and used my free time to write a 1500 Word essay titled ‘Should Zero Be considered a Number?’ However, it is the statistics and probability area that my fascination heavily lies, evident in my result of 96 UMS points in the AQA Statistics exam. It is, primarily, the most important application of mathematical concepts to real-life situations. In particular, I enjoy carrying out Chi-square tests to determine any association between two variables. This is because of its complicated process, and the need to identify the necessary use of Yates’ correction, or the grouping of data too small, to obtain accurate results. I find a great sense of achievement on completion of these tests, as well as many other processes studied in statistics. The fact that a large part of Actuarial Science involves analysing statistical data, needed to assess the future effects of large financial risks, is what draws me to the degree. I understand the Actuary profession is not an easy one, but one that requires dedication and motivation, something I have proven to be great qualities of mine. Since the age of 15, I have had at least one job at any time, holding two part-time jobs whilst taking my A-levels; with my results proving my handling of this to have been successful. As a part-time receptionist for three years, from the age of 15, I have developed strong communication and interpersonal skills. This will enable me to effectively convey my knowledge of complex financial information to non-specialists, essential for someone entering the Actuarial profession. My attraction to the degree, as well as my suitability to the career is clear. It is my desire to learn and my constant search for a challenge that draws me to this path. I thrive on spontaneity, and knowing of the diverse and wide-ranging activities an Actuary can find themselves responsible for in their day-to-day work, from analysing risk and calculating profit, to developing and overseeing new financial products, I find myself impatient to start my studies in Actuarial Science. In the meantime, I plan to spend the year keeping up to date with current world financial affairs and to take work experience where possible, so that I am thoroughly prepared to begin a successful Actuarial career path in 2014. 13 Did you know...  The starting salary of actuarial graduates is on average upwards of £30,000.  Our course is accredited by the Institute and Faculty of Actuaries for the purpose of exemption from some professional examinations.</t>
-        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
+        <v>1002</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>I am currently taking A-levels in History, English Language and Literature, and Geography. I enjoy all of these subjects but History has always stood out as my favourite. As part of my History AS-level studies, I undertook an American History unit. Learning about the Civil Rights Movement and the events which caused it really captured my imagination and sparked an interest in the USA, which grew after studying The Crucible in my English Literature course. America’s rich and controversial history, and its sociology, such as the existence of an ‘American Dream’ are so different from our own English history and heritage; it is this contrast which fascinates me. I have attended a number of university open days in which I listened to sample lectures and talks about American Studies. The diversity of American Studies appeals to me greatly, and the flexibility of the subject allows me to develop my existing interests in history, literature and sociology. I would also like the opportunity to study another aspect of American Studies, such as politics. British and American politics have always interested me, but A-level Politics was not available as an option at my school. At school, I am involved in the Debating Team, and we have had several achievements. Most recently, we came second in the inter-school county finals, the topic being ‘Do stop-and-search tactics erode civil liberties?’. Other topics we have debated include abortion, ID cards and the Scottish Referendum. Debating compliments my interests in history and politics and I look forward to continuing this pursuit at university. I played hockey for my school until year 10, and I am also a Sixth Form prefect. This responsibility involves helping teachers in lessons and disciplining the younger students in corridors. I also have a weekend job waitressing in a local restaurant. My friends are very important to me, and I enjoy spending time with them. My sister attends the University of Essex, and I have visited her twice. This has given me a flavour of student life and as a result I feel I would fit in well at university. Overall, I am looking forward to going to university and particularly to furthering my interest in American Studies.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BSC C354 AMERICAN STUDIES</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AMERICAN STUDIES</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
         <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>AMERICAN STUDIES</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>I am currently taking A-levels in History, English Language and Literature, and Geography. I enjoy all of these subjects but History has always stood out as my favourite. As part of my History AS-level studies, I undertook an American History unit. Learning about the Civil Rights Movement and the events which caused it really captured my imagination and sparked an interest in the USA, which grew after studying The Crucible in my English Literature course. America’s rich and controversial history, and its sociology, such as the existence of an ‘American Dream’ are so different from our own English history and heritage; it is this contrast which fascinates me. I have attended a number of university open days in which I listened to sample lectures and talks about American Studies. The diversity of American Studies appeals to me greatly, and the flexibility of the subject allows me to develop my existing interests in history, literature and sociology. I would also like the opportunity to study another aspect of American Studies, such as politics. British and American politics have always interested me, but A-level Politics was not available as an option at my school. At school, I am involved in the Debating Team, and we have had several achievements. Most recently, we came second in the inter-school county finals, the topic being ‘Do stop-and-search tactics erode civil liberties?’. Other topics we have debated include abortion, ID cards and the Scottish Referendum. Debating compliments my interests in history and politics and I look forward to continuing this pursuit at university. I played hockey for my school until year 10, and I am also a Sixth Form prefect. This responsibility involves helping teachers in lessons and disciplining the younger students in corridors. I also have a weekend job waitressing in a local restaurant. My friends are very important to me, and I enjoy spending time with them. My sister attends the University of Essex, and I have visited her twice. This has given me a flavour of student life and as a result I feel I would fit in well at university. Overall, I am looking forward to going to university and particularly to furthering my interest in American Studies.</t>
-        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>My childhood visits to London always involved an excursion to a gallery or museum. The works of art that I saw there prompted me to ask many questions which sparked my lifelong interest in the visual arts: Why was the beautiful lady floating in a river full of flowers? Why was a whole lobster sitting on a telephone? Why did the Virgin Mary always seem to be wearing blue? As a child it was fun to try to answer the questions myself, but I only realised that art history existed as a subject in its own right when I chose to study Art at A-level. The critical and contextual studies element of the course helped me to realise many answers to my questions and showed me the varied ways in which the images which held my attention could act to document the times in which they were made. A single work could be inspired or sourced by anything and everything from literature, to history, religion, politics, or perhaps philosophies and economics; every single work of art had such diversity of meaning and a real ‘history’ of its own. So, the ‘beautiful lady floating in a river full of flowers’ seen through my eyes as a child is actually Sir John Everett Millais’ own version of Shakespeare’s ‘Ophelia’ the tragic heroine drowned as a result of her madness. More literally, it is the artist and model Lizzie Siddal, lover of Dante Gabriel Rossetti, posed in a bath in an antique dress. On a more historical level it is a ground breaking masterpiece by a Victorian rebel determined to paint with a truth to nature for him not seen since the work of the early Italian Masters. After my gap year, which was spent travelling in Europe and visiting my family in Spain, I have recently been working as a Saturday girl in my local John Lewis store. Although there is much routine sales work involved in the job, my keen eye for design detail, colour and an obvious flair for arrangement has already been noted. My counter supervisor often asks me to help arrange various display stands of perfumery and makeup, and also asks for my comments on the ways in which these can be made most appealing. I feel that even as a junior member of the team I am able to use my creativity to good effect, and use the skills that my love of the visual arts has helped to foster. In so doing I can work effectively and efficiently to help increase our counter sales. I have many interests including crafting and decoupage, and lots of my spare time is occupied making cards and small gifts for sale at local craft fairs. Often I have been lucky enough to sell everything that I have produced and also to generate some additional orders! Art History appeals to me not only because I love the visual arts but also because I would like to study a subject which can dovetail with so many others. I like the idea that I will eventually have a wide ranging vocational degree in a humanities subject which offers me the broadest possible scope with which to address my future career choices.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BSC W571 ART HISTORY</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ART HISTORY</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ART HISTORY</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>My childhood visits to London always involved an excursion to a gallery or museum. The works of art that I saw there prompted me to ask many questions which sparked my lifelong interest in the visual arts: Why was the beautiful lady floating in a river full of flowers? Why was a whole lobster sitting on a telephone? Why did the Virgin Mary always seem to be wearing blue? As a child it was fun to try to answer the questions myself, but I only realised that art history existed as a subject in its own right when I chose to study Art at A-level. The critical and contextual studies element of the course helped me to realise many answers to my questions and showed me the varied ways in which the images which held my attention could act to document the times in which they were made. A single work could be inspired or sourced by anything and everything from literature, to history, religion, politics, or perhaps philosophies and economics; every single work of art had such diversity of meaning and a real ‘history’ of its own. So, the ‘beautiful lady floating in a river full of flowers’ seen through my eyes as a child is actually Sir John Everett Millais’ own version of Shakespeare’s ‘Ophelia’ the tragic heroine drowned as a result of her madness. More literally, it is the artist and model Lizzie Siddal, lover of Dante Gabriel Rossetti, posed in a bath in an antique dress. On a more historical level it is a ground breaking masterpiece by a Victorian rebel determined to paint with a truth to nature for him not seen since the work of the early Italian Masters. After my gap year, which was spent travelling in Europe and visiting my family in Spain, I have recently been working as a Saturday girl in my local John Lewis store. Although there is much routine sales work involved in the job, my keen eye for design detail, colour and an obvious flair for arrangement has already been noted. My counter supervisor often asks me to help arrange various display stands of perfumery and makeup, and also asks for my comments on the ways in which these can be made most appealing. I feel that even as a junior member of the team I am able to use my creativity to good effect, and use the skills that my love of the visual arts has helped to foster. In so doing I can work effectively and efficiently to help increase our counter sales. I have many interests including crafting and decoupage, and lots of my spare time is occupied making cards and small gifts for sale at local craft fairs. Often I have been lucky enough to sell everything that I have produced and also to generate some additional orders! Art History appeals to me not only because I love the visual arts but also because I would like to study a subject which can dovetail with so many others. I like the idea that I will eventually have a wide ranging vocational degree in a humanities subject which offers me the broadest possible scope with which to address my future career choices.</t>
-        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>When I was twelve years old the car that my mother was driving was hit by lorry. Thankfully she recovered from the accident but only because she had a blood transfusion. Since that dreadful day I have aimed for a career in transfusion science because without skilled biomedical scientists, the blood transfusion service would collapse. With such a clear focus on my chosen career, I have been able to do extensive research into the skills and attributes that a biomedical scientist must possess. I am focused and determined, and am both accurate and efficient. These skills are essential because patient’s lives and the treatment of illnesses depend upon me. I am also confident that my choice of A- and AS-levels, Biology, Chemistry, Psychology and Maths, will provide me with the solid foundation needed to proceed to undergraduate level. The practical side of biology and chemistry has enabled me to gain good laboratory skills and I am eager to acquire more developed and sophisticated techniques at university. Maths has helped me to think logically and to develop my understanding of numerical information. Psychology has improved my written communication skills, which I believe to be important for any subject at university. Throughout my school career I have enjoyed positions of considerable responsibility. I was nominated form captain four years running and elected Head Girl during my final year. This was a demanding job as I was required to represent the school at prestigious events and do a lot of public speaking (something which used to scare me greatly). At our GCSE prize giving I received prizes for biology and maths. I was also awarded the Stubbs Cup which I am extremely proud of. I love spending time in the country walking my greyhounds Mollie and Vinnie. I have taken Mollie to many open shows and am hoping to present her at her first championship show this Christmas. Showing and caring for dogs involves discipline and attention to detail. It is also a great way to socialise as I am constantly meeting new faces at the weekly club I attend. I can’t wait to start university because I will get the opportunity to meet people from all over the world. When I’m not walking the dog’s I can be found in the gym. I like keeping fit and look forward to trying new sports and activities at university. I have also recently started working at the gym in their crèche. I enjoy working with children and have attained my first aid certificate. I think that being a biomedical scientist will be a rewarding career because I will be doing work that will help improve people’s health and cure diseases. University has been my goal for a long time now and I look forward to the challenge ahead of me.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BSC D655 BIOCHEMISTRY AND BIOMEDICAL SCIENCE</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BIOCHEMISTRY AND BIOMEDICAL SCIENCE</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
         <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>BIOCHEMISTRY AND BIOMEDICAL SCIENCE</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>When I was twelve years old the car that my mother was driving was hit by lorry. Thankfully she recovered from the accident but only because she had a blood transfusion. Since that dreadful day I have aimed for a career in transfusion science because without skilled biomedical scientists, the blood transfusion service would collapse. With such a clear focus on my chosen career, I have been able to do extensive research into the skills and attributes that a biomedical scientist must possess. I am focused and determined, and am both accurate and efficient. These skills are essential because patient’s lives and the treatment of illnesses depend upon me. I am also confident that my choice of A- and AS-levels, Biology, Chemistry, Psychology and Maths, will provide me with the solid foundation needed to proceed to undergraduate level. The practical side of biology and chemistry has enabled me to gain good laboratory skills and I am eager to acquire more developed and sophisticated techniques at university. Maths has helped me to think logically and to develop my understanding of numerical information. Psychology has improved my written communication skills, which I believe to be important for any subject at university. Throughout my school career I have enjoyed positions of considerable responsibility. I was nominated form captain four years running and elected Head Girl during my final year. This was a demanding job as I was required to represent the school at prestigious events and do a lot of public speaking (something which used to scare me greatly). At our GCSE prize giving I received prizes for biology and maths. I was also awarded the Stubbs Cup which I am extremely proud of. I love spending time in the country walking my greyhounds Mollie and Vinnie. I have taken Mollie to many open shows and am hoping to present her at her first championship show this Christmas. Showing and caring for dogs involves discipline and attention to detail. It is also a great way to socialise as I am constantly meeting new faces at the weekly club I attend. I can’t wait to start university because I will get the opportunity to meet people from all over the world. When I’m not walking the dog’s I can be found in the gym. I like keeping fit and look forward to trying new sports and activities at university. I have also recently started working at the gym in their crèche. I enjoy working with children and have attained my first aid certificate. I think that being a biomedical scientist will be a rewarding career because I will be doing work that will help improve people’s health and cure diseases. University has been my goal for a long time now and I look forward to the challenge ahead of me.</t>
-        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>From an early age I have been fascinated by biology. I can clearly recall spending time in the garden with my Grandfather looking at bugs and creepy crawlies. As I grew up my affinity with the natural world developed and studying biology at university is the next step on my journey. I have had the most amazing gap year experience protecting the Lora turtles of Costa Rica from human poachers and beach erosion. As a volunteer on the programme I was able to help with research and conservation work such as night patrolling, working in the hatcheries, collecting eggs, rescuing and tagging turtles and helping the baby turtles get to the sea! This opportunity has enabled me to grow as a person in many ways. It certainly has been the best preparation possible for university life, as I have acquired all kinds of skills that will be essential for a new life away from friends and family. A-level Biology has certainly provided me with an excellent grounding and I am confident that I have a real aptitude for this challenging discipline. I have enjoyed all of the modules taken so far, especially ecosystems as we had to consider the dynamics of such systems and look into human activities that impact on them. I particularly like doing practical work and look forward to being able to gain experience with more developed pieces of apparatus at university. I have held several positions of responsibility. During my final year at school I was appointed to the position of Senior Prefect. This was a great honour and I learnt many new skills, including public speaking. At college I continued this type of responsibility by being nominated Student Voice Rep. This position required me to attend various meetings with different types of people including the Board of Governors. I was the voice for all 2,000 students at our college. I am an eager table tennis player and regularly compete at county level. I find it to be an excellent form of exercise for the body and mind! I am keen to try out different sports when I reach university because it will be the perfect way to make new friends and stay healthy. The Duke of Edinburgh Award Scheme is also something that I am involved in and I have completed bronze, silver and gold awards. I am hoping to be involved in promoting the award scheme to young people in the future as I have really benefited from it and would like to be able to share my experience with others.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BSC S281 BIOLOGICAL SCIENCES</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BIOLOGICAL SCIENCES</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
         <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>BIOLOGICAL SCIENCES</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>From an early age I have been fascinated by biology. I can clearly recall spending time in the garden with my Grandfather looking at bugs and creepy crawlies. As I grew up my affinity with the natural world developed and studying biology at university is the next step on my journey. I have had the most amazing gap year experience protecting the Lora turtles of Costa Rica from human poachers and beach erosion. As a volunteer on the programme I was able to help with research and conservation work such as night patrolling, working in the hatcheries, collecting eggs, rescuing and tagging turtles and helping the baby turtles get to the sea! This opportunity has enabled me to grow as a person in many ways. It certainly has been the best preparation possible for university life, as I have acquired all kinds of skills that will be essential for a new life away from friends and family. A-level Biology has certainly provided me with an excellent grounding and I am confident that I have a real aptitude for this challenging discipline. I have enjoyed all of the modules taken so far, especially ecosystems as we had to consider the dynamics of such systems and look into human activities that impact on them. I particularly like doing practical work and look forward to being able to gain experience with more developed pieces of apparatus at university. I have held several positions of responsibility. During my final year at school I was appointed to the position of Senior Prefect. This was a great honour and I learnt many new skills, including public speaking. At college I continued this type of responsibility by being nominated Student Voice Rep. This position required me to attend various meetings with different types of people including the Board of Governors. I was the voice for all 2,000 students at our college. I am an eager table tennis player and regularly compete at county level. I find it to be an excellent form of exercise for the body and mind! I am keen to try out different sports when I reach university because it will be the perfect way to make new friends and stay healthy. The Duke of Edinburgh Award Scheme is also something that I am involved in and I have completed bronze, silver and gold awards. I am hoping to be involved in promoting the award scheme to young people in the future as I have really benefited from it and would like to be able to share my experience with others.</t>
-        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>I have always been a very academically determined and studious individual, hence why I knew that a degree at university would be my definite next step. I have a broad interest in many subject areas but feel drawn towards a business-orientated degree. Coming from the background of a small family business, I have been inspired by my parents and am keen to gain the essential skills to expand our growing empire! I am very aware that today’s business requires not just balancing the books; it is about the investment and the management of assets, people, opportunities and risk. I am confident that studying a business degree at university level will prepare me well for my future ahead. A-level Business Studies has definitely provided me with a solid foundation which I am eager to develop. ‘Management, Culture and Communication’ is the module that interested me the most this year and I have undertaken extensive further reading in my own time. When in Rome or Rio of Riyadh: Cultural Q&amp;As for successful Business Behaviour around the World by Gwyneth Oloffson, is an excellent read. I particularly enjoyed her views on manners and gift giving across the world. Studying A-level Psychology has also given me insight into the human influences on organisational behaviour through looking at motivational theories, such as the hierarchy of needs model proposed by Maslow. The coursework element has developed my skills in collecting and analysing data in order to establish trends and draw conclusions. A-level English Language has allowed me to develop an ability to express my ideas clearly and concisely. I have a wide circle of friends and we often meet in our village pub to compete in the quiz. I also enjoy playing football with friends and hope to join a team when I arrive at university. Our family business is very important to me and I work most weekends at our shop, often shadowing my father at meetings with suppliers. I take work very seriously and I feel that my conscientious approach will stand me in good stead for university study. I recently attended a two-day Challenge of Management conference at my local university. I also had the chance to go on a tour given by a current student and this made me realise that a campus-style university is definitely suited to me. I am certainly going to take advantage of all the opportunities that universities provide to widen your knowledge like clubs and societies.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BSC B250 BUSINESS AND MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BUSINESS AND MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
         <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>BUSINESS AND MANAGEMENT</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>I have always been a very academically determined and studious individual, hence why I knew that a degree at university would be my definite next step. I have a broad interest in many subject areas but feel drawn towards a business-orientated degree. Coming from the background of a small family business, I have been inspired by my parents and am keen to gain the essential skills to expand our growing empire! I am very aware that today’s business requires not just balancing the books; it is about the investment and the management of assets, people, opportunities and risk. I am confident that studying a business degree at university level will prepare me well for my future ahead. A-level Business Studies has definitely provided me with a solid foundation which I am eager to develop. ‘Management, Culture and Communication’ is the module that interested me the most this year and I have undertaken extensive further reading in my own time. When in Rome or Rio of Riyadh: Cultural Q&amp;As for successful Business Behaviour around the World by Gwyneth Oloffson, is an excellent read. I particularly enjoyed her views on manners and gift giving across the world. Studying A-level Psychology has also given me insight into the human influences on organisational behaviour through looking at motivational theories, such as the hierarchy of needs model proposed by Maslow. The coursework element has developed my skills in collecting and analysing data in order to establish trends and draw conclusions. A-level English Language has allowed me to develop an ability to express my ideas clearly and concisely. I have a wide circle of friends and we often meet in our village pub to compete in the quiz. I also enjoy playing football with friends and hope to join a team when I arrive at university. Our family business is very important to me and I work most weekends at our shop, often shadowing my father at meetings with suppliers. I take work very seriously and I feel that my conscientious approach will stand me in good stead for university study. I recently attended a two-day Challenge of Management conference at my local university. I also had the chance to go on a tour given by a current student and this made me realise that a campus-style university is definitely suited to me. I am certainly going to take advantage of all the opportunities that universities provide to widen your knowledge like clubs and societies.</t>
-        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B9" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>I am fascinated by the way developments in computer science have changed our lives and our work. The world-wide computing industry is set to continue evolving and I am determined to be part of this. Since a very early age I enjoyed playing with computers and now that I am at college I spend a lot of time working with them. As well as Computing, I am taking A-levels in Physics and Mathematics. I believe that these disciplines compliment each other brilliantly and will prepare me well for undergraduate study. A major recent achievement has been a GCSE physics revision site which I designed for the students at my school. I carried out a significant amount of research prior to designing the site and this was definitely a worthwhile activity. This made me realise how important communication is when producing products. My main goal is to be part of a team that creates efficient and useful software for consumers. My interest in computing has not only been restricted to school. With the help of my Dad, I have used all of my knowledge and skill to set up my own computer-related business. This challenge has given me a totally new perspective on how IT businesses operate. I had to write a business plan which was a totally alien experience for me, but once completed and implemented I was rewarded with the satisfaction of knowing that I had achieved something that most people would never have the chance to do, especially at my age. Although computers are my passion I still enjoy many other activities, particularly reading. Science fiction author Theodore Sturgeon wrote, “a good science fiction story is a story about human beings, with a human problem, and a human solution, that would not have happened at all without its science content”; science fiction is certainly the genre I like most probably because of the link between science and real-life. When I’m not reading I can usually be found at the swimming pool. I have swum competitively since the age of nine. I hope to continue swimming at university and intend to start water-polo, as this is something which I tried at a recent summer school and loved. I look forward to extending my knowledge of computers and believe that university will enhance the opportunities that I have ahead of me.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BSC B330 COMPUTER SCIENCE</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>COMPUTER SCIENCE</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
         <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>COMPUTER SCIENCE</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>I am fascinated by the way developments in computer science have changed our lives and our work. The world-wide computing industry is set to continue evolving and I am determined to be part of this. Since a very early age I enjoyed playing with computers and now that I am at college I spend a lot of time working with them. As well as Computing, I am taking A-levels in Physics and Mathematics. I believe that these disciplines compliment each other brilliantly and will prepare me well for undergraduate study. A major recent achievement has been a GCSE physics revision site which I designed for the students at my school. I carried out a significant amount of research prior to designing the site and this was definitely a worthwhile activity. This made me realise how important communication is when producing products. My main goal is to be part of a team that creates efficient and useful software for consumers. My interest in computing has not only been restricted to school. With the help of my Dad, I have used all of my knowledge and skill to set up my own computer-related business. This challenge has given me a totally new perspective on how IT businesses operate. I had to write a business plan which was a totally alien experience for me, but once completed and implemented I was rewarded with the satisfaction of knowing that I had achieved something that most people would never have the chance to do, especially at my age. Although computers are my passion I still enjoy many other activities, particularly reading. Science fiction author Theodore Sturgeon wrote, “a good science fiction story is a story about human beings, with a human problem, and a human solution, that would not have happened at all without its science content”; science fiction is certainly the genre I like most probably because of the link between science and real-life. When I’m not reading I can usually be found at the swimming pool. I have swum competitively since the age of nine. I hope to continue swimming at university and intend to start water-polo, as this is something which I tried at a recent summer school and loved. I look forward to extending my knowledge of computers and believe that university will enhance the opportunities that I have ahead of me.</t>
-        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
+        <v>1008</v>
+      </c>
+      <c r="B10" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>From an early age I have always been fascinated by the stage. Far from being mere entertainment, I believe that a theatrical production can convey so much information and emotion to the audience. Although my main experience in theatre to date is through acting, I am also very interested in other aspects of productions such as lighting and set design, and am keen to learn more about this in a university degree. For my GCSE Drama final production, a group of us produced a play based on a short story by A.L. Kennedy. Because there were only six of us in the group, we shared a lot of responsibility. I played one of the main characters and was also in charge of obtaining the props we needed. These tasks were enjoyable but the most challenging part of the production was to adapt the story for the stage, and produce a script as close to the original story as possible. This was a demanding but enjoyable job and really opened my eyes to the complexity of adapting stories to the stage. As well as Theatre Studies, my other AS-levels are in English Literature, Sociology and Biology. In English Literature we have just completed a module on plays in which we studied Death of a Salesman by Arthur Miller and Shakespeare’s Henry V. I go to the theatre as often as I can, and have seen many amateur and professional productions. My favourite playwright is Willy Russell. I think all his plays provide an interesting social commentary, and successfully blend comedy and tragedy. I have seen many musicals, but Blood Brothers is by far my favourite; I have now seen it four times! I am looking forward to discovering more playwrights while at university. My interest in drama and the theatre takes up a lot of my social life. I have taken part in all my school’s productions and am also involved in a local drama group ‘The Bournemouth and Boscombe Light Operatic Club’ - BBLOC for short. Every year we hold a major production, the most recent being Oh What a Lovely War. I value the experience of being part of this group as I get to work with people of all different ages. I also have a part-time job in a local Beefeater restaurant. This job has taught me the value of being able to work as part of a team, and I think helps me improve my performance within BBLOC and at school, as good teamwork is crucial to a successful production. I am looking forward to joining a drama society at university, and also possibly a film society, as the cinema and films are another of my passions. I feel I have a lot to contribute to university life and hope you will consider me for a place at your University.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BSC P958 DRAMA</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>DRAMA</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
         <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>DRAMA</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>From an early age I have always been fascinated by the stage. Far from being mere entertainment, I believe that a theatrical production can convey so much information and emotion to the audience. Although my main experience in theatre to date is through acting, I am also very interested in other aspects of productions such as lighting and set design, and am keen to learn more about this in a university degree. For my GCSE Drama final production, a group of us produced a play based on a short story by A.L. Kennedy. Because there were only six of us in the group, we shared a lot of responsibility. I played one of the main characters and was also in charge of obtaining the props we needed. These tasks were enjoyable but the most challenging part of the production was to adapt the story for the stage, and produce a script as close to the original story as possible. This was a demanding but enjoyable job and really opened my eyes to the complexity of adapting stories to the stage. As well as Theatre Studies, my other AS-levels are in English Literature, Sociology and Biology. In English Literature we have just completed a module on plays in which we studied Death of a Salesman by Arthur Miller and Shakespeare’s Henry V. I go to the theatre as often as I can, and have seen many amateur and professional productions. My favourite playwright is Willy Russell. I think all his plays provide an interesting social commentary, and successfully blend comedy and tragedy. I have seen many musicals, but Blood Brothers is by far my favourite; I have now seen it four times! I am looking forward to discovering more playwrights while at university. My interest in drama and the theatre takes up a lot of my social life. I have taken part in all my school’s productions and am also involved in a local drama group ‘The Bournemouth and Boscombe Light Operatic Club’ - BBLOC for short. Every year we hold a major production, the most recent being Oh What a Lovely War. I value the experience of being part of this group as I get to work with people of all different ages. I also have a part-time job in a local Beefeater restaurant. This job has taught me the value of being able to work as part of a team, and I think helps me improve my performance within BBLOC and at school, as good teamwork is crucial to a successful production. I am looking forward to joining a drama society at university, and also possibly a film society, as the cinema and films are another of my passions. I feel I have a lot to contribute to university life and hope you will consider me for a place at your University.</t>
-        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
+        <v>1009</v>
+      </c>
+      <c r="B11" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Since starting my AS-level studies in Economics, I have been eager to continue to a higher level. I am particularly interested in the behaviour of firms and organisations from an economic point of view and I have focused my coursework in this field. I regularly read newspapers and economic publications such as The Economist to keep up-to-date with developments in the field, and I find it easy to use my mathematical and analytical skills to apply different economic theories to a range of real-life economic situations. I also take Maths and Politics at AS-level and know that the skills I am acquiring from these will prepare me well for university- level study. I recently enjoyed the chance to put some of my business economic theory into practice when I took part in an economics and business project called Young Enterprise. With a group of peers I set up a small company and sold stationery packs to students at our school. It was an excellent experience and I was able to enhance my management, communication and teamwork skills. I also achieved a distinction in the associated exam. I would consider myself to be a very hard worker both in and out of school. Since the age of 16 I have worked part-time at Tescos and have enjoyed positions of increasing responsibility. I now co-ordinate a small group of staff on the shopfloor and have leant a lot about the way businesses operate in the real world. I would be keen to continue working part-time within this company while at university, as I know I would be able to manage my time succesffully and would enjoy being self sufficient. I have a real passion for all kinds of sport and regularly represent my school in various activities ranging from tennis to football. I have played tennis at county-level for two years now and am looking forward to trying new sports at university. Music is also very important to me and I am a member of the sixth form rock band ‘Chaos’. I am thrilled at the prospect of facing new challenges, including working and living independently. I also believe that I will gain a highly marketable set of skills from the study of economics at university, which will prepare me well for the exciting future ahead. Did you know...  Essex is top 25 for Economics (The Times and Sunday Times Good University Guide 2021).</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>BSC Q404 ECONOMICS</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ECONOMICS</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
         <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>ECONOMICS</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Since starting my AS-level studies in Economics, I have been eager to continue to a higher level. I am particularly interested in the behaviour of firms and organisations from an economic point of view and I have focused my coursework in this field. I regularly read newspapers and economic publications such as The Economist to keep up-to-date with developments in the field, and I find it easy to use my mathematical and analytical skills to apply different economic theories to a range of real-life economic situations. I also take Maths and Politics at AS-level and know that the skills I am acquiring from these will prepare me well for university- level study. I recently enjoyed the chance to put some of my business economic theory into practice when I took part in an economics and business project called Young Enterprise. With a group of peers I set up a small company and sold stationery packs to students at our school. It was an excellent experience and I was able to enhance my management, communication and teamwork skills. I also achieved a distinction in the associated exam. I would consider myself to be a very hard worker both in and out of school. Since the age of 16 I have worked part-time at Tescos and have enjoyed positions of increasing responsibility. I now co-ordinate a small group of staff on the shopfloor and have leant a lot about the way businesses operate in the real world. I would be keen to continue working part-time within this company while at university, as I know I would be able to manage my time succesffully and would enjoy being self sufficient. I have a real passion for all kinds of sport and regularly represent my school in various activities ranging from tennis to football. I have played tennis at county-level for two years now and am looking forward to trying new sports at university. Music is also very important to me and I am a member of the sixth form rock band ‘Chaos’. I am thrilled at the prospect of facing new challenges, including working and living independently. I also believe that I will gain a highly marketable set of skills from the study of economics at university, which will prepare me well for the exciting future ahead. Did you know...  Essex is top 25 for Economics (The Times and Sunday Times Good University Guide 2021).</t>
-        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
+        <v>1010</v>
+      </c>
+      <c r="B12" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>My interest in linguistics has grown from my first year of sixth form when I took a course in English Language. During this course, I studied the work of Trudgill. I found this particularly interesting as I enjoyed looking at how and why the social class of a person affects how they speak. I also found the gender and language issues relating to how males and females approach language in a different manner very interesting. I have a general interest in sociology and look forward to combining this with my interests in linguistics. Last summer I spent a month in Spain where I worked as a teaching assistant in a local school. Working in a foreign country allowed me to experience life where I did not completely understand the language used around me. It became clear that language is an essential tool used everyday for communication. This opportunity allowed me to see language being used in different environments and I now want to understand how languages are used and how they work. During my time at school I have been actively involved with the netball team, working my way to becoming captain last year. Being involved in the team has allowed me to develop my communication and time-management skills, along with motivating the rest of my team. I really enjoy volunteering and once a week I help younger students to learn Spanish. After my undergraduate degree I plan to study a PGCE as I would like to become a secondary school teacher of Spanish. I believe that volunteering will allow me to learn skills which will help me with this career path. I have also been the Managing Director of a Young Enterprise company which won two awards for quality and best product at the local awards evening. Our company has also been selected to attend the regional awards later this month. From this interesting experience I learnt a lot about how the real world works and I worked incredibly hard to achieve my highest potential and compete successfully. As well as these school organised activities, I also work in the local supermarket. I have to relate to the customers and assist them in a variety of ways. I feel this has boosted my confidence and improved my inter-personal skills both of which I think will help me in the transition from sixth form to university. I believe that studying linguistics at university will expand my knowledge of language, which I know will be essential in my future career. I look forward to setting myself new challenges and building upon my existing experience, which will hopefully help me to achieve my ambition of becoming a successful teacher.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>BSC D101 ENGLISH LANGUAGE AND LINGUISTICS</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ENGLISH LANGUAGE AND LINGUISTICS</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
         <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>ENGLISH LANGUAGE AND LINGUISTICS</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>My interest in linguistics has grown from my first year of sixth form when I took a course in English Language. During this course, I studied the work of Trudgill. I found this particularly interesting as I enjoyed looking at how and why the social class of a person affects how they speak. I also found the gender and language issues relating to how males and females approach language in a different manner very interesting. I have a general interest in sociology and look forward to combining this with my interests in linguistics. Last summer I spent a month in Spain where I worked as a teaching assistant in a local school. Working in a foreign country allowed me to experience life where I did not completely understand the language used around me. It became clear that language is an essential tool used everyday for communication. This opportunity allowed me to see language being used in different environments and I now want to understand how languages are used and how they work. During my time at school I have been actively involved with the netball team, working my way to becoming captain last year. Being involved in the team has allowed me to develop my communication and time-management skills, along with motivating the rest of my team. I really enjoy volunteering and once a week I help younger students to learn Spanish. After my undergraduate degree I plan to study a PGCE as I would like to become a secondary school teacher of Spanish. I believe that volunteering will allow me to learn skills which will help me with this career path. I have also been the Managing Director of a Young Enterprise company which won two awards for quality and best product at the local awards evening. Our company has also been selected to attend the regional awards later this month. From this interesting experience I learnt a lot about how the real world works and I worked incredibly hard to achieve my highest potential and compete successfully. As well as these school organised activities, I also work in the local supermarket. I have to relate to the customers and assist them in a variety of ways. I feel this has boosted my confidence and improved my inter-personal skills both of which I think will help me in the transition from sixth form to university. I believe that studying linguistics at university will expand my knowledge of language, which I know will be essential in my future career. I look forward to setting myself new challenges and building upon my existing experience, which will hopefully help me to achieve my ambition of becoming a successful teacher.</t>
-        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
+        <v>1011</v>
+      </c>
+      <c r="B13" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>(example of a joint degree application) The history, politics and culture of the European Union, since its beginnings in the 1950s, has always interested me, and as a result European Studies is a natural choice of degree for me to study. I find Europe fasinating: that a group of diverse countries with their own cultures and heritage should come together and form common policies is an interesting and often controversial area, and one I would like to discover more about. I have chosen to apply for a joint course in European Studies and Politics as I believe the two disciplines are closely interlinked. Politics plays such a major part in all our lives and the work of governments shapes both the life of the individual and a country’s place on the word stage. Through my A-level History scheme I have studied British governments in the nineteenth and twentieth centrury and I also keep up-to-date with modern UK and foreign politics by watching the news and reading broadsheet newspapers. I am particularly drawn to European Studies and Politics as the degree would offer me the opportunity to become familiar with the political systems of several countries; I am looking forward to studying more of the history and politics of Europe, particularly in the twentieth century. As well as History, my other two A-levels are Business Studies and German. I also have an AS-level in Performing Arts. In Business Studies my main interest is the relationship between governments and industry; how, for example, the laws passed by governments can shape the present and future industry of a country. This relationship will be the topic for my final project in Business Studies. I have travelled to France, Spain and Germany several times, for family holidays and for exchange trips with my school. I am looking forward to the year abroad offered by the degree and would like to spend that in Germany or France. Outside of school I play the trumpet and cornet, and am currently working toward my grade 6 exam for the trumpet. I have played in several school concerts and am a member of the Watchet Town Brass Band. I also enjoy going to the cinema and spending time with my friends. I am looking forward to the opportunities that going to university will provide and to studying two subjects that have always fasinated me. I have a long-term goal of working abroad, possibly for the EU in Brussels, and I hope with a university education behind me, I can be successful in this mission.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>BSC F202 EUROPEAN STUDIES AND POLITICS</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>EUROPEAN STUDIES AND POLITICS</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
         <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>EUROPEAN STUDIES AND POLITICS</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>(example of a joint degree application) The history, politics and culture of the European Union, since its beginnings in the 1950s, has always interested me, and as a result European Studies is a natural choice of degree for me to study. I find Europe fasinating: that a group of diverse countries with their own cultures and heritage should come together and form common policies is an interesting and often controversial area, and one I would like to discover more about. I have chosen to apply for a joint course in European Studies and Politics as I believe the two disciplines are closely interlinked. Politics plays such a major part in all our lives and the work of governments shapes both the life of the individual and a country’s place on the word stage. Through my A-level History scheme I have studied British governments in the nineteenth and twentieth centrury and I also keep up-to-date with modern UK and foreign politics by watching the news and reading broadsheet newspapers. I am particularly drawn to European Studies and Politics as the degree would offer me the opportunity to become familiar with the political systems of several countries; I am looking forward to studying more of the history and politics of Europe, particularly in the twentieth century. As well as History, my other two A-levels are Business Studies and German. I also have an AS-level in Performing Arts. In Business Studies my main interest is the relationship between governments and industry; how, for example, the laws passed by governments can shape the present and future industry of a country. This relationship will be the topic for my final project in Business Studies. I have travelled to France, Spain and Germany several times, for family holidays and for exchange trips with my school. I am looking forward to the year abroad offered by the degree and would like to spend that in Germany or France. Outside of school I play the trumpet and cornet, and am currently working toward my grade 6 exam for the trumpet. I have played in several school concerts and am a member of the Watchet Town Brass Band. I also enjoy going to the cinema and spending time with my friends. I am looking forward to the opportunities that going to university will provide and to studying two subjects that have always fasinated me. I have a long-term goal of working abroad, possibly for the EU in Brussels, and I hope with a university education behind me, I can be successful in this mission.</t>
-        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
+        <v>1012</v>
+      </c>
+      <c r="B14" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Film Studies is my chosen subject at University because I have a lifelong passion for all aspects of film. Obviously I love watching and critiquing films, but I also have an interest in film production, including special effects. I enjoy seeing the new developments in CGI and other techniques such as prosthetics, sound, and camera angles. As a child I loved Disney films but as I have matured I have grown to enjoy the works of David Lynch and to appreciate European cinema. The film which has had the most impact upon me in recent years is Florian Hankel von Donnersmarck’s ‘The Lives of Others’. As I am also interested in modern European history I found this film compelling and raised many questions in my mind. Much of my interest in film stems from my A-level work in Media Studies. I have written several long essays which have achieved good marks, and have taught me the importance of expressing an argument clearly, and paying attention to detail. Taking Media Studies has opened my eyes to film interpretation and the film making approach, such as the use of story boards and editing techniques. I enjoy making and producing films as much as interpreting them. My most recent piece of coursework was a short promotional film designed to encourage children to play tennis. Although the production was at times challenging, as there were some complicated shots to film and the ‘stars’ of our film were all under nine years old, it was very rewarding to see the finished result and it received great praise. I really look forward to making and producing films at university. My other A-level courses are History and Business Studies. I also took AS-level German which has helped in my appreciation of European cinema. I look forward to the opportunity to perhaps continue some aspects of these courses at University. I am also keen to get involved with the University Film Society, and also the football and tennis teams. Sport is a big part of my life, both as an active player and a spectator. I have been fortunate to be able to travel around Europe to attend tennis tournaments and have seen many of the ‘greats’ play: Roger Federer and Rafael Nadal to name a few. My all time idol is Pete Sampras; I admired his combination of huge talent and commitment which made him, in my opinion, one of the best tennis players of all time. I am looking forward to the opportunities a university degree will give me, both academic and social and I feel ready for this new chapter in my life. Through my studies and my personal experiences, I am convinced that Film Studies is the right choice for my university degree.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>BSC R480 FILM STUDIES</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>FILM STUDIES</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
         <v>13</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>FILM STUDIES</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Film Studies is my chosen subject at University because I have a lifelong passion for all aspects of film. Obviously I love watching and critiquing films, but I also have an interest in film production, including special effects. I enjoy seeing the new developments in CGI and other techniques such as prosthetics, sound, and camera angles. As a child I loved Disney films but as I have matured I have grown to enjoy the works of David Lynch and to appreciate European cinema. The film which has had the most impact upon me in recent years is Florian Hankel von Donnersmarck’s ‘The Lives of Others’. As I am also interested in modern European history I found this film compelling and raised many questions in my mind. Much of my interest in film stems from my A-level work in Media Studies. I have written several long essays which have achieved good marks, and have taught me the importance of expressing an argument clearly, and paying attention to detail. Taking Media Studies has opened my eyes to film interpretation and the film making approach, such as the use of story boards and editing techniques. I enjoy making and producing films as much as interpreting them. My most recent piece of coursework was a short promotional film designed to encourage children to play tennis. Although the production was at times challenging, as there were some complicated shots to film and the ‘stars’ of our film were all under nine years old, it was very rewarding to see the finished result and it received great praise. I really look forward to making and producing films at university. My other A-level courses are History and Business Studies. I also took AS-level German which has helped in my appreciation of European cinema. I look forward to the opportunity to perhaps continue some aspects of these courses at University. I am also keen to get involved with the University Film Society, and also the football and tennis teams. Sport is a big part of my life, both as an active player and a spectator. I have been fortunate to be able to travel around Europe to attend tennis tournaments and have seen many of the ‘greats’ play: Roger Federer and Rafael Nadal to name a few. My all time idol is Pete Sampras; I admired his combination of huge talent and commitment which made him, in my opinion, one of the best tennis players of all time. I am looking forward to the opportunities a university degree will give me, both academic and social and I feel ready for this new chapter in my life. Through my studies and my personal experiences, I am convinced that Film Studies is the right choice for my university degree.</t>
-        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
+        <v>1013</v>
+      </c>
+      <c r="B15" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>I am applying to study History at university because this is a subject which has fascinated me from an early age. The study of history plays a large part in understanding who we are today, how nations are shaped, how conflicts begin and how they are resolved, and most importantly, how a country’s heritage and values are created. My GCSE and A-level syllabi have concentrated heavily on modern British history, an era which fascinates me, and which I would like to continue studying at university. In my spare time I have been reading into British immigration in the 1950s, a topic I find very interesting and a subject particularly relevant to present-day Britain. I have also been interested in military history, in particular the use of animals in warfare, especially homing pigeons and horses. This interest culminated in me going to see the play ‘War Horse’ by Michael Morpurgo, which left a great impression upon me. This link between past and present is one which fascinates me. I have been to several museums and historical sites, and am a member of English Heritage. I find that visiting historical sites is a great complement to my studies. I am passionate about preserving historical buildings as they serve to remind us of our country’s past. As well as studying British history at university, I also look forward to studying the history of other countries as a comparison to our own, such as Russian or American history. To relax from my studies I play rugby in my school team: we were recently finalists in an inter-school tournament. I also work weekends in my local Asda store, where I have recently been promoted to ‘greeter’. This is a front-of-house job where I help customers with queries and make announcements over the loudspeaker system. I also watch out for suspicious activity and recently helped to catch a notorious shoplifter who was later arrested and charged. Being a greeter has improved my confidence greatly and taught me how to think on my feet and handle responsibility. I am looking forward to going to university as it will provide me with an opportunity to be independent and to meet new people. But most importantly, I am looking forward to furthering my knowledge of history and continuing my interest in what has always been my favourite subject.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BSC C627 HISTORY</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>HISTORY</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
         <v>14</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>HISTORY</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>I am applying to study History at university because this is a subject which has fascinated me from an early age. The study of history plays a large part in understanding who we are today, how nations are shaped, how conflicts begin and how they are resolved, and most importantly, how a country’s heritage and values are created. My GCSE and A-level syllabi have concentrated heavily on modern British history, an era which fascinates me, and which I would like to continue studying at university. In my spare time I have been reading into British immigration in the 1950s, a topic I find very interesting and a subject particularly relevant to present-day Britain. I have also been interested in military history, in particular the use of animals in warfare, especially homing pigeons and horses. This interest culminated in me going to see the play ‘War Horse’ by Michael Morpurgo, which left a great impression upon me. This link between past and present is one which fascinates me. I have been to several museums and historical sites, and am a member of English Heritage. I find that visiting historical sites is a great complement to my studies. I am passionate about preserving historical buildings as they serve to remind us of our country’s past. As well as studying British history at university, I also look forward to studying the history of other countries as a comparison to our own, such as Russian or American history. To relax from my studies I play rugby in my school team: we were recently finalists in an inter-school tournament. I also work weekends in my local Asda store, where I have recently been promoted to ‘greeter’. This is a front-of-house job where I help customers with queries and make announcements over the loudspeaker system. I also watch out for suspicious activity and recently helped to catch a notorious shoplifter who was later arrested and charged. Being a greeter has improved my confidence greatly and taught me how to think on my feet and handle responsibility. I am looking forward to going to university as it will provide me with an opportunity to be independent and to meet new people. But most importantly, I am looking forward to furthering my knowledge of history and continuing my interest in what has always been my favourite subject.</t>
-        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
+        <v>1014</v>
+      </c>
+      <c r="B16" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>My name is Katherine Jones and I am 17 years old. I am applying to study Latin American Studies at university as I am passionate about other countries and cultures and I would relish the opportunity to study the development of other cultures in more depth at university. I have an interest in all of the developing world, but Latin America has always particularly fascinated me. It has a rich history and vibrant culture and the countries that make up Latin America are so diverse. I closely follow the news and current affairs of Latin America, such as the re-election of Michelle Bachelet in 2014, Chile’s first female president and the relationship between Cuba and the United States. I am also fascinated by the region’s geography and how that has affected the fortunes of its countries. It has always been my ambition to travel to Peru to visit the ancient Inca civilisations. I intend to take a gap year before starting university and plan to travel to Chile with Teaching and Projects Abroad. I am really looking forward to this experience as a chance to see first-hand the culture of a Latin American country and an opportunity to improve my Spanish! I also hope to travel to neighbouring countries and believe that spending my gap year in Latin America will surely enhance my study of the region at degree level. I currently attend a large sixth form college, which is very different to the small rural school I went to previously. The college environment requires me to be more independent and motivate myself to study, and I have met hundreds of new people and made new friends. As a result I feel I will adapt to a university community well. At college I write articles for the monthly newsletter and help with campaigns such as boycotting Nestle products in the college canteen and running petitions on behalf of Amnesty International. I feel strongly about human rights abuse around the world and would like to continue my work for Amnesty while at university. I have attended a number of university open days and feel I will adapt to university life well. I believe I have the passion and commitment to make a success of my studies at university, and I am greatly looking forward to the opportunity of studying Latin America in more depth.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>BSC E664 LATIN AMERICAN STUDIES</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LATIN AMERICAN STUDIES</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
         <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>LATIN AMERICAN STUDIES</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>My name is Katherine Jones and I am 17 years old. I am applying to study Latin American Studies at university as I am passionate about other countries and cultures and I would relish the opportunity to study the development of other cultures in more depth at university. I have an interest in all of the developing world, but Latin America has always particularly fascinated me. It has a rich history and vibrant culture and the countries that make up Latin America are so diverse. I closely follow the news and current affairs of Latin America, such as the re-election of Michelle Bachelet in 2014, Chile’s first female president and the relationship between Cuba and the United States. I am also fascinated by the region’s geography and how that has affected the fortunes of its countries. It has always been my ambition to travel to Peru to visit the ancient Inca civilisations. I intend to take a gap year before starting university and plan to travel to Chile with Teaching and Projects Abroad. I am really looking forward to this experience as a chance to see first-hand the culture of a Latin American country and an opportunity to improve my Spanish! I also hope to travel to neighbouring countries and believe that spending my gap year in Latin America will surely enhance my study of the region at degree level. I currently attend a large sixth form college, which is very different to the small rural school I went to previously. The college environment requires me to be more independent and motivate myself to study, and I have met hundreds of new people and made new friends. As a result I feel I will adapt to a university community well. At college I write articles for the monthly newsletter and help with campaigns such as boycotting Nestle products in the college canteen and running petitions on behalf of Amnesty International. I feel strongly about human rights abuse around the world and would like to continue my work for Amnesty while at university. I have attended a number of university open days and feel I will adapt to university life well. I believe I have the passion and commitment to make a success of my studies at university, and I am greatly looking forward to the opportunity of studying Latin America in more depth.</t>
-        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
+        <v>1015</v>
+      </c>
+      <c r="B17" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>My aspration to study law is firmly rooted in my interest in world events and with my desire to help others. Law affects our everyday lives, almost without us noticing. The news always features an aspect of law up for debate. Ethical issues are often brought to the forefront on topics such as animal testing, abortion and gay rights. I find these debates absolutely fascinating and the complexity of law continues to astound me. I have always maintained an independent, self- motivated approach to my academic studies. Having studied a broad range of AS and A-level subjects, I feel I have acquired a strong selection of skills: from Mathematics and Philosophy I have learnt the art of questioning the world around us and developing a keen sense of intellectual curiosity; from English Language and General Studies I have understood the importance of expressing myself clearly and concisely through words; whilst from ICT I have developed a solid understanding of an area which is playing an increasingly important role in today’s society. I have spent time in the public galleries of both the local County Court and High Court. I am fascinated by the processes that take place and my long-term ambition is to play an integral role in the court room. In November I am due to shadow a district judge for a week, giving valuable insight into the day to day workings of the job. I built upon my initial interest by keenly reading The Law Machine by Marcel Berlins and Clare Dyer; it provided me with a firm grounding in the essential principles of the British legal system and highlighted its apparent weaknesses. To gain a different perspective of the law I had the chance to take a work experience placement with a local solicitor’s firm. My work evolved from basic administrative duties, such as filing, faxing and answering telephone calls, into accompanying solicitors to court and liaising with barristers on behalf of the firm. The opportunity to work alongside people who have dedicated their lives to the law has strengthened my decision to study this challenging discipline. A keen passion of mine is debating and I have represented my school in various competitions. In year eleven I was a member of the winning team in the Rotary Youth Speaks final for East Anglia. Our presentation – Is it ever justifiable to execute criminals? – was given a special award of distinction. I was appointed senior prefect at my school this year and it is a position which I take great pride in. It involves helping to maintain discipline amongst the younger pupils during lunch-breaks and representing the school at various events. In my spare time I like to swim and play netball. Although I do not play at a recognised level, I would be very keen to continue them as hobbies when I reach university. I understand the importance of having a good balance between work and play and I am confident that I would make the most of my time as a student. I believe that my ability to motivate myself is a key factor in my overall success. I am an extremely hardworking person and I am committed to reaching my goals. I believe I can contribute a genuine passion and enthusiasm for reading law and I thank you for taking the time to consider my application.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BSC G625 LAW AND HUMAN RIGHTS</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LAW AND HUMAN RIGHTS</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
         <v>16</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>LAW AND HUMAN RIGHTS</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>My aspration to study law is firmly rooted in my interest in world events and with my desire to help others. Law affects our everyday lives, almost without us noticing. The news always features an aspect of law up for debate. Ethical issues are often brought to the forefront on topics such as animal testing, abortion and gay rights. I find these debates absolutely fascinating and the complexity of law continues to astound me. I have always maintained an independent, self- motivated approach to my academic studies. Having studied a broad range of AS and A-level subjects, I feel I have acquired a strong selection of skills: from Mathematics and Philosophy I have learnt the art of questioning the world around us and developing a keen sense of intellectual curiosity; from English Language and General Studies I have understood the importance of expressing myself clearly and concisely through words; whilst from ICT I have developed a solid understanding of an area which is playing an increasingly important role in today’s society. I have spent time in the public galleries of both the local County Court and High Court. I am fascinated by the processes that take place and my long-term ambition is to play an integral role in the court room. In November I am due to shadow a district judge for a week, giving valuable insight into the day to day workings of the job. I built upon my initial interest by keenly reading The Law Machine by Marcel Berlins and Clare Dyer; it provided me with a firm grounding in the essential principles of the British legal system and highlighted its apparent weaknesses. To gain a different perspective of the law I had the chance to take a work experience placement with a local solicitor’s firm. My work evolved from basic administrative duties, such as filing, faxing and answering telephone calls, into accompanying solicitors to court and liaising with barristers on behalf of the firm. The opportunity to work alongside people who have dedicated their lives to the law has strengthened my decision to study this challenging discipline. A keen passion of mine is debating and I have represented my school in various competitions. In year eleven I was a member of the winning team in the Rotary Youth Speaks final for East Anglia. Our presentation – Is it ever justifiable to execute criminals? – was given a special award of distinction. I was appointed senior prefect at my school this year and it is a position which I take great pride in. It involves helping to maintain discipline amongst the younger pupils during lunch-breaks and representing the school at various events. In my spare time I like to swim and play netball. Although I do not play at a recognised level, I would be very keen to continue them as hobbies when I reach university. I understand the importance of having a good balance between work and play and I am confident that I would make the most of my time as a student. I believe that my ability to motivate myself is a key factor in my overall success. I am an extremely hardworking person and I am committed to reaching my goals. I believe I can contribute a genuine passion and enthusiasm for reading law and I thank you for taking the time to consider my application.</t>
-        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
+        <v>1016</v>
+      </c>
+      <c r="B18" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>I am applying to study Liberal Arts at university because I have always been interested in many different subjects and reluctant to pinpoint a favourite. When I first heard that there was a degree that covered a range of different disciplines I realised that this would be the perfect option for me. During my sixth form studies I was always aware that I wanted to attend university but, unlike my friends, I found it difficult to find a university course which was not totally specialised and would allow me to continue with my wide range of interests. The huge range of disciplines available in the Liberal Arts course is a perfect fit for my wide ranging interests and thirst for many different types of knowledge, and I am convinced it is the best course choice for me. While studying for my International Baccalaureate, the courses I enjoyed the most were English, Philosophy, French and History. These are all subjects I am interested in continuing at university, particularly English Literature. I was also fortunate to take standard level Latin which has provided a useful background for my interests in languages and philosophy. Since I left school two years ago, I have worked in several places: in the retail sector and more recently in an art gallery owned by a family friend. Working full time has opened my eyes to the world of work and taught me skills which I believe will be invaluable at university: time management, responsibility, interacting with all walks of life and the importance of being friendly and cheerful to others. While working in the gallery I have also been given additional roles and responsibilities: such as organising exhibitions, managing the mailing list and publicising the gallery. I recently had to organise a private view for a local artist which involved printing invitations, organising the guest list and refreshments, and ensuring the evening ran smoothly. I really enjoyed this experience and I am now considering a career in gallery management or public relations. I also enjoy reading (my favourite genres are the historical novel and autobiographies) and travelling: I am currently saving in order to spend a month travelling around Europe this summer. I am looking forward to meeting lots of different people and enjoying the cultural diversity that a university will have to offer. But more importantly, I am keen to return to academic life and will relish the challenges that a broad-ranging degree such as Liberal Arts will have to offer me.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BSC K319 LIBERAL ARTS</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LIBERAL ARTS</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
         <v>17</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>LIBERAL ARTS</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>I am applying to study Liberal Arts at university because I have always been interested in many different subjects and reluctant to pinpoint a favourite. When I first heard that there was a degree that covered a range of different disciplines I realised that this would be the perfect option for me. During my sixth form studies I was always aware that I wanted to attend university but, unlike my friends, I found it difficult to find a university course which was not totally specialised and would allow me to continue with my wide range of interests. The huge range of disciplines available in the Liberal Arts course is a perfect fit for my wide ranging interests and thirst for many different types of knowledge, and I am convinced it is the best course choice for me. While studying for my International Baccalaureate, the courses I enjoyed the most were English, Philosophy, French and History. These are all subjects I am interested in continuing at university, particularly English Literature. I was also fortunate to take standard level Latin which has provided a useful background for my interests in languages and philosophy. Since I left school two years ago, I have worked in several places: in the retail sector and more recently in an art gallery owned by a family friend. Working full time has opened my eyes to the world of work and taught me skills which I believe will be invaluable at university: time management, responsibility, interacting with all walks of life and the importance of being friendly and cheerful to others. While working in the gallery I have also been given additional roles and responsibilities: such as organising exhibitions, managing the mailing list and publicising the gallery. I recently had to organise a private view for a local artist which involved printing invitations, organising the guest list and refreshments, and ensuring the evening ran smoothly. I really enjoyed this experience and I am now considering a career in gallery management or public relations. I also enjoy reading (my favourite genres are the historical novel and autobiographies) and travelling: I am currently saving in order to spend a month travelling around Europe this summer. I am looking forward to meeting lots of different people and enjoying the cultural diversity that a university will have to offer. But more importantly, I am keen to return to academic life and will relish the challenges that a broad-ranging degree such as Liberal Arts will have to offer me.</t>
-        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
+        <v>1017</v>
+      </c>
+      <c r="B19" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>“Every secret of a writer’s soul, every experience of his life, every quality of his mind is written large in his works.” This quote by Virginia Woolf summarises why I believe literature to be so fascinating and why I have chosen English Literature as the subject I wish to study at university level. Through my studies of A-level English Language and Literature, and my own discoveries of authors such as Virginia Woolf, George Eliot and Charles Dickens, I have found that authors do more than just tell a story; they also convey their own personal thoughts and opinions, and often provide a fascinating social commentary. For example, Middlemarch gives a snapshot of nineteenth century provincial life, while Jane Austen’s novels often reveal her own – sometimes sarcastic – views on social situations in the early nineteenth century. These are the reasons why I believe literature to be such a rich source of information and why I would really like to study English Literature in more depth at undergraduate level. I spent my schools work experience week as an assistant in my local ‘Borders’ bookshop. I enjoyed working with the staff on book promotions and helping to organise a book signing which was taking place the following week. I was also asked to write reviews on books I had read which were then displayed on the shelves. As I have a passion for books and reading, I really enjoyed encouraging others – particularly children – who visited the shop to read more, or to discover authors they had perhaps not previously heard of. Although I am not longer convinced that working in retail is right for me, after university I would like to pursue a career involving books and literature, such as perhaps publishing or teaching English. As well as reading, I also enjoy getting involved in my local community in my spare time. As part of my school’s voluntering scheme, I work on Wednesday afternoons in a local charity shop. Through this work I have become friendly with some of the older ladies who work in the shop and now help them to write our village newsletter, which is distributed monthly. This is an interesting and satisfying task. As I enjoy reading and discovering new writers and what they have to say about the world, I feel that English Literature is the right degree choice for me. I am looking forward to the opportunities I will have to discuss and write about texts, and the increased career prospects I am sure being a graduate will offer me.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>BSC D788 LITERATURE AND CREATIVE WRITING</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LITERATURE AND CREATIVE WRITING</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
         <v>18</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>LITERATURE AND CREATIVE WRITING</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>“Every secret of a writer’s soul, every experience of his life, every quality of his mind is written large in his works.” This quote by Virginia Woolf summarises why I believe literature to be so fascinating and why I have chosen English Literature as the subject I wish to study at university level. Through my studies of A-level English Language and Literature, and my own discoveries of authors such as Virginia Woolf, George Eliot and Charles Dickens, I have found that authors do more than just tell a story; they also convey their own personal thoughts and opinions, and often provide a fascinating social commentary. For example, Middlemarch gives a snapshot of nineteenth century provincial life, while Jane Austen’s novels often reveal her own – sometimes sarcastic – views on social situations in the early nineteenth century. These are the reasons why I believe literature to be such a rich source of information and why I would really like to study English Literature in more depth at undergraduate level. I spent my schools work experience week as an assistant in my local ‘Borders’ bookshop. I enjoyed working with the staff on book promotions and helping to organise a book signing which was taking place the following week. I was also asked to write reviews on books I had read which were then displayed on the shelves. As I have a passion for books and reading, I really enjoyed encouraging others – particularly children – who visited the shop to read more, or to discover authors they had perhaps not previously heard of. Although I am not longer convinced that working in retail is right for me, after university I would like to pursue a career involving books and literature, such as perhaps publishing or teaching English. As well as reading, I also enjoy getting involved in my local community in my spare time. As part of my school’s voluntering scheme, I work on Wednesday afternoons in a local charity shop. Through this work I have become friendly with some of the older ladies who work in the shop and now help them to write our village newsletter, which is distributed monthly. This is an interesting and satisfying task. As I enjoy reading and discovering new writers and what they have to say about the world, I feel that English Literature is the right degree choice for me. I am looking forward to the opportunities I will have to discuss and write about texts, and the increased career prospects I am sure being a graduate will offer me.</t>
-        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
+        <v>1018</v>
+      </c>
+      <c r="B20" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mathematics is a subject that I have thoroughly enjoyed throughout my primary and secondary education. I enjoy the challenge of thinking in a logical way and am always attracted to mathematical problems, however difficult and regardless of the form in which they come. Having studied A-level Mathematics for a year, I have been able to have a taste of many different topics. Pure mathematics is my favourite area, particularly sequences and functions, and I look forward to learning more about these and other topics in much more depth. A Mathematics degree will provide me with the challenge that I am ready for. I always work hard at school and have a good level of concentration. I am efficient and make good use of the time from free periods to complete my homework. Deadlines are always met to the best of my ability and I make a real effort to present my work clearly. As a member of my school community, I believe that I have contributed greatly. Having been appointed to the position of Head Maths Prefect, I am now responsible for the Maths Department during lunchtimes and run a weekly maths club called Pythagoras. This club is for younger years and I set logic puzzles, help with homework and hold a quiz at the end of the session. Spending time with the younger pupils has made me realise that I might like to be a teacher. My enthusiasm for the subject resulted in me winning a maths prize, which was a great honour. Out of school I am a keen musician and play trumpet in a brass band. I have been a member for almost four years and would like to continue this interest at university. I am due to take my grade 8 exam this winter and intend to start teaching afterwards as I think this would be a valuable skill. Another passion of mine is comic art. John McLusky, who was the original artist of the James Bond 007 Strip Cartoon Series in the Daily Express, is my hero, and I enjoy visiting his exhibitions whenever I can. I am greatly looking forward to the transition from school to university because of the independence and opportunities that university life will offer. I will get involved in many different clubs and societies and try some new sports, like karate, that I am not able to do at school. I believe that the challenge of studying and developing my mathematical knowledge to a higher level is going to be one that I will thoroughly enjoy. Did you know...  89% of our maths students are in employment or further study (Graduate Outcomes 2020).</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>BSC B470 MATHEMATICS</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>MATHEMATICS</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
         <v>19</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>MATHEMATICS</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Mathematics is a subject that I have thoroughly enjoyed throughout my primary and secondary education. I enjoy the challenge of thinking in a logical way and am always attracted to mathematical problems, however difficult and regardless of the form in which they come. Having studied A-level Mathematics for a year, I have been able to have a taste of many different topics. Pure mathematics is my favourite area, particularly sequences and functions, and I look forward to learning more about these and other topics in much more depth. A Mathematics degree will provide me with the challenge that I am ready for. I always work hard at school and have a good level of concentration. I am efficient and make good use of the time from free periods to complete my homework. Deadlines are always met to the best of my ability and I make a real effort to present my work clearly. As a member of my school community, I believe that I have contributed greatly. Having been appointed to the position of Head Maths Prefect, I am now responsible for the Maths Department during lunchtimes and run a weekly maths club called Pythagoras. This club is for younger years and I set logic puzzles, help with homework and hold a quiz at the end of the session. Spending time with the younger pupils has made me realise that I might like to be a teacher. My enthusiasm for the subject resulted in me winning a maths prize, which was a great honour. Out of school I am a keen musician and play trumpet in a brass band. I have been a member for almost four years and would like to continue this interest at university. I am due to take my grade 8 exam this winter and intend to start teaching afterwards as I think this would be a valuable skill. Another passion of mine is comic art. John McLusky, who was the original artist of the James Bond 007 Strip Cartoon Series in the Daily Express, is my hero, and I enjoy visiting his exhibitions whenever I can. I am greatly looking forward to the transition from school to university because of the independence and opportunities that university life will offer. I will get involved in many different clubs and societies and try some new sports, like karate, that I am not able to do at school. I believe that the challenge of studying and developing my mathematical knowledge to a higher level is going to be one that I will thoroughly enjoy. Did you know...  89% of our maths students are in employment or further study (Graduate Outcomes 2020).</t>
-        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
+        <v>1019</v>
+      </c>
+      <c r="B21" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>‘If you can speak three languages, you are trilingual; if you can speak two languages, you are bilingual; if you can speak one language, you are English’. This German joke is one which I find amusing but also slightly shocking. Learning languages has always been a passion for me and it is my ambition to be fluent in at least one other language. This is why the decision to study Modern Languages at university was an easy choice to make. The ability to speak foreign languages and the privilege of communicating with others in their own language has always fascinated me. My mother’s side of the family is Welsh and one of my earliest memories was being upset that my cousins were speaking a mysterious language which I could not understand. I find it frustrating not to be able to communicate with others through a common language and I believe that by studying Modern Languages at university I will be helping to enrich my career prospects and gain invaluable skills I will use for the rest of my life. I am currently studying for A2 Levels in French, Spanish and Art. I enjoy all my subjects, and they challenge me in different ways. I am keen to continue my studies in French and Spanish at university, and I would also like to take up a third language such as Italian or Russian. The history and culture of Spain and France also interests me. In my AS studies, I researched the Spanish civil war and how it was reflected in pieces of art such as Picasso’s Guernica. In French I also wrote an extended essay on how the region of Brittany was once a separate country with its own language and customs, and drew parallels between Brittany and Cornwall. I believe that my language studies will be enriched by also studying the history and culture of the countries where these languages are spoken and look forward to learning more about France and Spain at university. I plan to take a gap year before starting university and have been researching into organisations which offer placements teaching English to children. I would like to go to a Latin American country, such as Chile or Brazil, so I could improve my Spanish. These plans tie in with my interest in language learning and I would like to share my passion for languages with others. In my spare time I play the piano and read. I also have a part-time job in a local café and babysit for several families in my village. I am looking forward to university as I believe it is the next step in my life and will help me reach my linguistic goals. Did you know...  We specialise in developing translation, interpreting and subtitling skills at undergraduate level using the latest technology in our multimedia labs.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>BSC K661 MODERN LANGUAGES</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>MODERN LANGUAGES</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
         <v>20</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>MODERN LANGUAGES</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>‘If you can speak three languages, you are trilingual; if you can speak two languages, you are bilingual; if you can speak one language, you are English’. This German joke is one which I find amusing but also slightly shocking. Learning languages has always been a passion for me and it is my ambition to be fluent in at least one other language. This is why the decision to study Modern Languages at university was an easy choice to make. The ability to speak foreign languages and the privilege of communicating with others in their own language has always fascinated me. My mother’s side of the family is Welsh and one of my earliest memories was being upset that my cousins were speaking a mysterious language which I could not understand. I find it frustrating not to be able to communicate with others through a common language and I believe that by studying Modern Languages at university I will be helping to enrich my career prospects and gain invaluable skills I will use for the rest of my life. I am currently studying for A2 Levels in French, Spanish and Art. I enjoy all my subjects, and they challenge me in different ways. I am keen to continue my studies in French and Spanish at university, and I would also like to take up a third language such as Italian or Russian. The history and culture of Spain and France also interests me. In my AS studies, I researched the Spanish civil war and how it was reflected in pieces of art such as Picasso’s Guernica. In French I also wrote an extended essay on how the region of Brittany was once a separate country with its own language and customs, and drew parallels between Brittany and Cornwall. I believe that my language studies will be enriched by also studying the history and culture of the countries where these languages are spoken and look forward to learning more about France and Spain at university. I plan to take a gap year before starting university and have been researching into organisations which offer placements teaching English to children. I would like to go to a Latin American country, such as Chile or Brazil, so I could improve my Spanish. These plans tie in with my interest in language learning and I would like to share my passion for languages with others. In my spare time I play the piano and read. I also have a part-time job in a local café and babysit for several families in my village. I am looking forward to university as I believe it is the next step in my life and will help me reach my linguistic goals. Did you know...  We specialise in developing translation, interpreting and subtitling skills at undergraduate level using the latest technology in our multimedia labs.</t>
-        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
+        <v>1020</v>
+      </c>
+      <c r="B22" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Philosophy involves a critical examination of our most fundamental beliefs about truth and reality, right and wrong. It challenges many of our assumptions about what we know and how we should live. It is for these reasons that Philosophy intrigues me more than any other discipline that I have studied. My teacher told me that the best reason for studying anything is if you enjoy it. I thoroughly enjoy Philosophy and know that I will have the determination to do well at university. A-level Philosophy has provided me with an excellent grounding on which to build. By reading Plato’s Republic I have become particularly intrigued by the field of ethics, and I am especially interested in the apparent conflict between causation and free will. This issue has profound significance to society and social justice, and the ways in which we choose to reward and punish. Psychology is another favourite subject which I am taking at A-level and I am definitely acquiring transferable skills which will assist me when I reach university. I enjoy music and gained a distinction in my grade 5 flute. I have also become involved with Worldwide Volunteers, an organisation which gives people volunteering placements across the world. So far I have done placements locally, mainly working in a care home organising activities for patients with dementia. I hope in the future to take up a volunteering placement further afield, such as in Africa. When I was a child, my family was based in several countries for my father’s work, and I feel lucky to have met many people from different cultures and backgrounds. These experiences have made me very aware that cultural diversity is a fantastic thing and I am very excited about meeting new people at university. Apart from academic study, I believe that university life will offer me a solid start in life generally and I am eager to become involved in such a large community. Did you know...  Philosophy graduates are well-suited to a wide range of occupations, including law, PR, journalism and the media, the Civil Service, charity work, banking, and the NHS.  We focus on the existential questions of human life, and provide a critical perspective on the social, political and economic challenges we are facing today by combining Anglo-American and European Continental philosophy.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>BSC L865 PHILOSOPHY</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>PHILOSOPHY</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
         <v>21</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>PHILOSOPHY</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Philosophy involves a critical examination of our most fundamental beliefs about truth and reality, right and wrong. It challenges many of our assumptions about what we know and how we should live. It is for these reasons that Philosophy intrigues me more than any other discipline that I have studied. My teacher told me that the best reason for studying anything is if you enjoy it. I thoroughly enjoy Philosophy and know that I will have the determination to do well at university. A-level Philosophy has provided me with an excellent grounding on which to build. By reading Plato’s Republic I have become particularly intrigued by the field of ethics, and I am especially interested in the apparent conflict between causation and free will. This issue has profound significance to society and social justice, and the ways in which we choose to reward and punish. Psychology is another favourite subject which I am taking at A-level and I am definitely acquiring transferable skills which will assist me when I reach university. I enjoy music and gained a distinction in my grade 5 flute. I have also become involved with Worldwide Volunteers, an organisation which gives people volunteering placements across the world. So far I have done placements locally, mainly working in a care home organising activities for patients with dementia. I hope in the future to take up a volunteering placement further afield, such as in Africa. When I was a child, my family was based in several countries for my father’s work, and I feel lucky to have met many people from different cultures and backgrounds. These experiences have made me very aware that cultural diversity is a fantastic thing and I am very excited about meeting new people at university. Apart from academic study, I believe that university life will offer me a solid start in life generally and I am eager to become involved in such a large community. Did you know...  Philosophy graduates are well-suited to a wide range of occupations, including law, PR, journalism and the media, the Civil Service, charity work, banking, and the NHS.  We focus on the existential questions of human life, and provide a critical perspective on the social, political and economic challenges we are facing today by combining Anglo-American and European Continental philosophy.</t>
-        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
+        <v>1021</v>
+      </c>
+      <c r="B23" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>I am eager to read Politics at university, particularly Comparative Politics and International Relations. I am currently studying History, Economics and English Literature at A-level. These subjects have enabled me to gain a selection of skills that I believe will prepare me well for a university degree. I am involved with the South Suffolk Liberal Democrats and have worked on many campaigns. I worked as a volunteer delivering leaflets and newsletters. I found this highly enjoyable and my ambition to become involved in real-life politics was confirmed. This has also increased my knowledge of the British political system. I enjoy becoming involved in debates. I have taken part in several on issues including the Scottish Referendum, capital punishment and the bedroom tax. This has developed my ability to form arguments and improved my public speaking skills. At the last general election my school held a mock election. I loved this experience and look forward to doing more things like this at university. I was recently involved in helping to organise a visit to my school by our local Labour MP, including a question-and-answer session with the students. This was followed by a visit to the Houses of Parliament in which we met with the MP again, and were also given the chance to watch a session of Prime Minister’s Question Time. This was interesting because it was at the time when many questions were being asked about the scandal surrounding expense claims submitted by MPs, and the ensuing debate was fascinating to watch. Dancing is my passion and I have been attending ballet, tap and modern classes since I was three years old. I was recently selected to attend a summer school at the Royal Ballet School. This was an excellent experience as I was chosen to play Juliet in the final show. I also work in a gift shop on Saturdays. My career ambition is to have a job in professional politics as an MP. I want to play a part in national policy making and legislation, as well as experiencing the pride of being a democratic representative of the people. I am excited by the prospect of becoming a student and relish the challenge ahead of me. Did you know...  The Government department is ranked among the top 30 departments in the QS World University Rankings (2020).  13th for Politics in the UK (The Times and Sunday Times Good University Guide 2021).</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>BSC B555 POLITICS</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>POLITICS</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
         <v>22</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>POLITICS</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>I am eager to read Politics at university, particularly Comparative Politics and International Relations. I am currently studying History, Economics and English Literature at A-level. These subjects have enabled me to gain a selection of skills that I believe will prepare me well for a university degree. I am involved with the South Suffolk Liberal Democrats and have worked on many campaigns. I worked as a volunteer delivering leaflets and newsletters. I found this highly enjoyable and my ambition to become involved in real-life politics was confirmed. This has also increased my knowledge of the British political system. I enjoy becoming involved in debates. I have taken part in several on issues including the Scottish Referendum, capital punishment and the bedroom tax. This has developed my ability to form arguments and improved my public speaking skills. At the last general election my school held a mock election. I loved this experience and look forward to doing more things like this at university. I was recently involved in helping to organise a visit to my school by our local Labour MP, including a question-and-answer session with the students. This was followed by a visit to the Houses of Parliament in which we met with the MP again, and were also given the chance to watch a session of Prime Minister’s Question Time. This was interesting because it was at the time when many questions were being asked about the scandal surrounding expense claims submitted by MPs, and the ensuing debate was fascinating to watch. Dancing is my passion and I have been attending ballet, tap and modern classes since I was three years old. I was recently selected to attend a summer school at the Royal Ballet School. This was an excellent experience as I was chosen to play Juliet in the final show. I also work in a gift shop on Saturdays. My career ambition is to have a job in professional politics as an MP. I want to play a part in national policy making and legislation, as well as experiencing the pride of being a democratic representative of the people. I am excited by the prospect of becoming a student and relish the challenge ahead of me. Did you know...  The Government department is ranked among the top 30 departments in the QS World University Rankings (2020).  13th for Politics in the UK (The Times and Sunday Times Good University Guide 2021).</t>
-        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
+        <v>1022</v>
+      </c>
+      <c r="B24" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>From an early age I have been interested in people and the way that they behave. This keen interest has been enhanced through my study of Psychology at A-level. I enjoy the variety of psychology and am eager to gain deeper knowledge and acquire practical skills in new areas of the discipline. My favourite module so far has been Social Psychology, with particular emphasis on physical attractiveness and the formation of relationships. My final-year project, ‘Do birds of a feather flock together?’ tests the hypothesis that people select partners who are of a similar level of attractiveness. I really like the way that you can apply different psychological theories to real-life situations. Although Psychology is my strongest subject, I have thoroughly enjoyed my other academic studies whilst at college and can appreciate how they will help me with my future studies. I have strengthened my assessment and evaluation skills through A-level Religious Studies, particularly the modules on philosophy and ethics. I believe that my study of ethics will be very advantageous when applied to the often problematic field of psychological research at university-level. I have achieved my Bronze Duke of Edinburgh Award, am currently working towards my Silver, and am hoping to gain Gold level at university. I love planning and undertaking expeditions as they are physically demanding and require total teamwork from start to finish. I also enjoy working for the ‘service’ element of the award. At the moment I visit the elderly residents at the local sheltered housing association once a week. This work can be quite emotionally draining at times but incredibly rewarding. At weekends I work in a restaurant and have recently been promoted to head waitress. This position means that I am in charge of four other waiting staff during service and am responsible for co-ordinating the weekly rota. People often comment that I possess good communication skills and that I am a real team- player. I know that these qualities will prepare me well for life at university. I am very determined to make the most of my time at university. I am looking forward to making lots of new friends and being able to get involved in different sporting and social activities. Although I don’t have any clear career plans, I know that a degree in psychology will provide me with an excellent set of transferrable skills for the future. Did you know...  91% of our psychology students are in employment or further study (Graduate Outcomes 2020).  You have unparalleled access to facilities such as EEG, TMS and eye tracking.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>BSC M153 PSYCHOLOGY</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>PSYCHOLOGY</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
         <v>23</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>PSYCHOLOGY</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>From an early age I have been interested in people and the way that they behave. This keen interest has been enhanced through my study of Psychology at A-level. I enjoy the variety of psychology and am eager to gain deeper knowledge and acquire practical skills in new areas of the discipline. My favourite module so far has been Social Psychology, with particular emphasis on physical attractiveness and the formation of relationships. My final-year project, ‘Do birds of a feather flock together?’ tests the hypothesis that people select partners who are of a similar level of attractiveness. I really like the way that you can apply different psychological theories to real-life situations. Although Psychology is my strongest subject, I have thoroughly enjoyed my other academic studies whilst at college and can appreciate how they will help me with my future studies. I have strengthened my assessment and evaluation skills through A-level Religious Studies, particularly the modules on philosophy and ethics. I believe that my study of ethics will be very advantageous when applied to the often problematic field of psychological research at university-level. I have achieved my Bronze Duke of Edinburgh Award, am currently working towards my Silver, and am hoping to gain Gold level at university. I love planning and undertaking expeditions as they are physically demanding and require total teamwork from start to finish. I also enjoy working for the ‘service’ element of the award. At the moment I visit the elderly residents at the local sheltered housing association once a week. This work can be quite emotionally draining at times but incredibly rewarding. At weekends I work in a restaurant and have recently been promoted to head waitress. This position means that I am in charge of four other waiting staff during service and am responsible for co-ordinating the weekly rota. People often comment that I possess good communication skills and that I am a real team- player. I know that these qualities will prepare me well for life at university. I am very determined to make the most of my time at university. I am looking forward to making lots of new friends and being able to get involved in different sporting and social activities. Although I don’t have any clear career plans, I know that a degree in psychology will provide me with an excellent set of transferrable skills for the future. Did you know...  91% of our psychology students are in employment or further study (Graduate Outcomes 2020).  You have unparalleled access to facilities such as EEG, TMS and eye tracking.</t>
-        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
+        <v>1023</v>
+      </c>
+      <c r="B25" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>I like the way that Sociology makes you question the world around you. For example, why do some people commit more crime than others? It was this question that sparked my interest in this discipline. During my AS-level studies I have had the opportunity to become familiar with various sociologists and their perspectives. I am particularly interested in the thoughts of Emile Durkheim in relation to crime and deviance. I am quite confident that when I graduate I would like to enter the police force, as my father and grandfather have done so before me. I have considered applying for a more focused criminology degree; however, I am attracted to the broad approach of a sociology degree and know that I will enjoy learning about all aspects of the discipline, not just crime. I also look forward to being able to acquire new skills within the area of research methods as I am able to appreciate the connection between theory and research. I also study Drama at AS-level and this has considerably increased my confidence as an actor over the past few years. My greatest dramatic achievement to date was performing in To Kill a Mocking Bird by Harper Lee earlier this year. I was selected to play the part of Atticus Finch and this was a fantastic experience. I had to work intensively with four people I didn’t usually associate with outside lessons, which greatly enhanced my communication and teamwork skills. The lengthy script that I had to commit to memory helped to further my confidence and self-belief. Another reason for enjoying this play is that it’s most important theme is the moral nature of human beings – that is, whether people are essentially good or essentially evil. I am a keen chess player and regularly compete in competitions at regional and national level. In 2013 I reached the finals of the UK Chess Challenge and that was without doubt the most pivotal moment in my chess-playing career. When I reach university I intend to get very involved in clubs and societies as I think this is an excellent way to socialise and develop your skills and hobbies. I work at the police station at the weekends doing administrative duties. This is an excellent opportunity as although I am not able to get quite as involved as I’d like, I am able to absorb information that will prepare me well for my future career. University life will suit me well because I am a sociable person who enjoys spending time with people. I am confident that I will be able to balance my studies with a healthy social life because I am organised and good at working to a timetable. Thank you for taking the time to read my application, I hope you can see my potential. Did you know...  Ranked 7th in the UK for Sociology in the QS World University Rankings by subject (2020).</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>BSC N631 SOCIOLOGY</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SOCIOLOGY</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
         <v>24</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>SOCIOLOGY</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>I like the way that Sociology makes you question the world around you. For example, why do some people commit more crime than others? It was this question that sparked my interest in this discipline. During my AS-level studies I have had the opportunity to become familiar with various sociologists and their perspectives. I am particularly interested in the thoughts of Emile Durkheim in relation to crime and deviance. I am quite confident that when I graduate I would like to enter the police force, as my father and grandfather have done so before me. I have considered applying for a more focused criminology degree; however, I am attracted to the broad approach of a sociology degree and know that I will enjoy learning about all aspects of the discipline, not just crime. I also look forward to being able to acquire new skills within the area of research methods as I am able to appreciate the connection between theory and research. I also study Drama at AS-level and this has considerably increased my confidence as an actor over the past few years. My greatest dramatic achievement to date was performing in To Kill a Mocking Bird by Harper Lee earlier this year. I was selected to play the part of Atticus Finch and this was a fantastic experience. I had to work intensively with four people I didn’t usually associate with outside lessons, which greatly enhanced my communication and teamwork skills. The lengthy script that I had to commit to memory helped to further my confidence and self-belief. Another reason for enjoying this play is that it’s most important theme is the moral nature of human beings – that is, whether people are essentially good or essentially evil. I am a keen chess player and regularly compete in competitions at regional and national level. In 2013 I reached the finals of the UK Chess Challenge and that was without doubt the most pivotal moment in my chess-playing career. When I reach university I intend to get very involved in clubs and societies as I think this is an excellent way to socialise and develop your skills and hobbies. I work at the police station at the weekends doing administrative duties. This is an excellent opportunity as although I am not able to get quite as involved as I’d like, I am able to absorb information that will prepare me well for my future career. University life will suit me well because I am a sociable person who enjoys spending time with people. I am confident that I will be able to balance my studies with a healthy social life because I am organised and good at working to a timetable. Thank you for taking the time to read my application, I hope you can see my potential. Did you know...  Ranked 7th in the UK for Sociology in the QS World University Rankings by subject (2020).</t>
-        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
+        <v>1024</v>
+      </c>
+      <c r="B26" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>I have always wanted a career in sport. Since taking A-level Sports Science my eyes have been opened to the opportunities that are available at undergraduate level. Detailed research has confirmed that a degree in Sports Science will provide me with a solid understanding of the biology, physiology and psychology required to succeed in my chosen discipline. I am fascinated by the various methods used to assess and measure physical activity and the changes in physiology that result from exercise and training. Last summer I attended a residential sports science summer school at my local university. We had various taster sessions with academics and I thoroughly enjoyed all of them. I was particularly fascinated by the Human Performance Unit because it was jam-packed with the latest gear. We were shown how all the different apparatus worked and were allowed to carry out tests using some of the more basic pieces. I also heard talks from current students and they really made me realise that I would fit into student life easily. Sport is obviously very important to me and I do get involved both in and out of school. I play hockey at county-level and will want to continue when I reach university. I am also eager to become involved in new sports and will enjoying helping to run clubs as I feel I have a lot of knowledge and experience to share. Football is also strong a passion of mine and I have recently been selected to assist with coaching the youth team at my town club. I am looking forward to working with children as I know that I will gain lots of new skills. I have a part-time job as a retail assistant in a leisure wear shop. I really enjoy helping customers and advising them on the most appropriate clothing and equipment. I am also responsible for the tills at the end of the day and am often trusted to close the shop. I would consider myself to be an excellent communicator and I also possess good time-keeping skills; I hate being late for anything! I know that both these attributes will stand me in good stead for academic life. I am so determined to become a student, studying the subject that I love. I know that I will put every effort into making the most of my time, both academically and socially.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>BSC P185 SPORTS AND EXERCISE SCIENCE AND SPORTS THERAPY</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SPORTS AND EXERCISE SCIENCE AND SPORTS THERAPY</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
         <v>25</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>SPORTS AND EXERCISE SCIENCE AND SPORTS THERAPY</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>I have always wanted a career in sport. Since taking A-level Sports Science my eyes have been opened to the opportunities that are available at undergraduate level. Detailed research has confirmed that a degree in Sports Science will provide me with a solid understanding of the biology, physiology and psychology required to succeed in my chosen discipline. I am fascinated by the various methods used to assess and measure physical activity and the changes in physiology that result from exercise and training. Last summer I attended a residential sports science summer school at my local university. We had various taster sessions with academics and I thoroughly enjoyed all of them. I was particularly fascinated by the Human Performance Unit because it was jam-packed with the latest gear. We were shown how all the different apparatus worked and were allowed to carry out tests using some of the more basic pieces. I also heard talks from current students and they really made me realise that I would fit into student life easily. Sport is obviously very important to me and I do get involved both in and out of school. I play hockey at county-level and will want to continue when I reach university. I am also eager to become involved in new sports and will enjoying helping to run clubs as I feel I have a lot of knowledge and experience to share. Football is also strong a passion of mine and I have recently been selected to assist with coaching the youth team at my town club. I am looking forward to working with children as I know that I will gain lots of new skills. I have a part-time job as a retail assistant in a leisure wear shop. I really enjoy helping customers and advising them on the most appropriate clothing and equipment. I am also responsible for the tills at the end of the day and am often trusted to close the shop. I would consider myself to be an excellent communicator and I also possess good time-keeping skills; I hate being late for anything! I know that both these attributes will stand me in good stead for academic life. I am so determined to become a student, studying the subject that I love. I know that I will put every effort into making the most of my time, both academically and socially.</t>
-        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
+        <v>1025</v>
+      </c>
+      <c r="B27" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>(example of a European application) Biomedical science has always interested me in both an educational and personal aspect. I believe that I will successfully complete this course, as I am extremely motivated and very willing to study, and learn new things in order to achieve my goals. The human body is incredibly interesting to me; the bones, veins, organs and the systems within this complex structure are a breath-taking design, and when examined in further detail the facts that are uncovered are even more fascinating. When I am in the laboratory I feel that I belong. I find that science subjects suit my inquisitive personality; I enjoy experimenting and understanding how the world works. This course will help me to achieve my dream career in IVF treatment and research. In my home country Cyprus, IVF is on the increase and it has a great potential for a career. I want to help couples, who are struggling to conceive. It will give me a great satisfaction that in the future I will be able to help them to change their lives in a good way. During my school years I have always been a top grade student in Chemistry, Physics and Biology. The experiments, which I did in my school Labs were successful and I enjoyed to work on them too much. My Projects were: Research in blood groups and Electrical systems for mobile homes. I also enjoyed being a part of science projects and competitions between schools and I always represented my school in the best possible way. I also took part in local and national science projects, which included research projects, experiments and I was also involved in the Lunar Eclipse Project, which was organised by our village. These gave me skills for research and presentation necessary for university life. I have been playing the Violin for the past 10 years. I took a part in various competitions and concerts as an individual and also as a part of an orchestra. I have also been an active volleyball player and a folk dancer since I was 10 years old. My volleyball team won numerous competitions and we also represented our team in Turkey with good results. I have also taken part in many festivals together with my folk dancing group. I entered a National Art competition, where I became third in Cyprus. I also enjoy reading books because I can learn new things and expand my horizons. During the science week, I was volunteered to go to the hospital together with my colleagues from school and with permission from patients we took their blood for research. It showed me how to deal with patients and how research should be done outside of the lab. It was a great experience for me and a quick glance into what I could be doing in my future career. I spent most of my weekends in my school laboratory, helping my teacher with projects. It gave me a lot of knowledge that would be useful for my future. One month after graduating from high school I entered an exam set by the European Union titled as `Discover Europe’ and won a full scholarship for an English language course in Brighton in the UK, where I am still studying. I want to carry on studying in the UK because I really love this country and its people who are friendly, warm and helpful towards me. I also like the multicultural environment in the UK where I can meet students from all over the World and see different cultures, nationalities and traditions.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>BSC Q173 BIOMEDICAL SCIENCE</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>BIOMEDICAL SCIENCE</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
         <v>26</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>BIOMEDICAL SCIENCE</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>(example of a European application) Biomedical science has always interested me in both an educational and personal aspect. I believe that I will successfully complete this course, as I am extremely motivated and very willing to study, and learn new things in order to achieve my goals. The human body is incredibly interesting to me; the bones, veins, organs and the systems within this complex structure are a breath-taking design, and when examined in further detail the facts that are uncovered are even more fascinating. When I am in the laboratory I feel that I belong. I find that science subjects suit my inquisitive personality; I enjoy experimenting and understanding how the world works. This course will help me to achieve my dream career in IVF treatment and research. In my home country Cyprus, IVF is on the increase and it has a great potential for a career. I want to help couples, who are struggling to conceive. It will give me a great satisfaction that in the future I will be able to help them to change their lives in a good way. During my school years I have always been a top grade student in Chemistry, Physics and Biology. The experiments, which I did in my school Labs were successful and I enjoyed to work on them too much. My Projects were: Research in blood groups and Electrical systems for mobile homes. I also enjoyed being a part of science projects and competitions between schools and I always represented my school in the best possible way. I also took part in local and national science projects, which included research projects, experiments and I was also involved in the Lunar Eclipse Project, which was organised by our village. These gave me skills for research and presentation necessary for university life. I have been playing the Violin for the past 10 years. I took a part in various competitions and concerts as an individual and also as a part of an orchestra. I have also been an active volleyball player and a folk dancer since I was 10 years old. My volleyball team won numerous competitions and we also represented our team in Turkey with good results. I have also taken part in many festivals together with my folk dancing group. I entered a National Art competition, where I became third in Cyprus. I also enjoy reading books because I can learn new things and expand my horizons. During the science week, I was volunteered to go to the hospital together with my colleagues from school and with permission from patients we took their blood for research. It showed me how to deal with patients and how research should be done outside of the lab. It was a great experience for me and a quick glance into what I could be doing in my future career. I spent most of my weekends in my school laboratory, helping my teacher with projects. It gave me a lot of knowledge that would be useful for my future. One month after graduating from high school I entered an exam set by the European Union titled as `Discover Europe’ and won a full scholarship for an English language course in Brighton in the UK, where I am still studying. I want to carry on studying in the UK because I really love this country and its people who are friendly, warm and helpful towards me. I also like the multicultural environment in the UK where I can meet students from all over the World and see different cultures, nationalities and traditions.</t>
-        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
+        <v>1026</v>
+      </c>
+      <c r="B28" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>(example of an international application) My first contact with English literature was at my high school. My English teacher showed us part of the movie Pride and Prejudice; I could not wait to watch the whole movie when I went home! After watching the movie several times, I tried to read the original book. At the time, I found the book difficult to understand, however the elegance and humour of the literature fascinated me deeply, and inspired me to find out more. I am looking forward to progressing my English ability and appreciating more excellent literary works in their original versions in the university. I enjoy reading masterpieces and watching classical movies. My huge interest in English is also influenced by my mother, who used to be a teacher and later founded a tutorial workshop teaching children English lessons. I therefore grew up amongst a group of children younger than me, who I would teach and support. Although it is hard work to teach others, I found that it was me who benefited most during the process. By helping these children, I would gain a deeper understanding and knowledge of the topic. Teaching has also enabled me to develop my communication skills and I feel satisfied helping others, whilst improving myself. With the support from my mother, I spent several months designing an English course to help children in China learn English; the course consists of 20 parts, including learning of the alphabet, grammar, and the practical application of language. Gradually, I found that my knowledge of English is not enough at all, just the tip of the iceberg, and I am passionate about finding out more. Through this process not only did I learn more English literature knowledge, but also fell in love with European culture and history. I got fine results in my courses including History, Geography and Politics, and ranked Top 5 in my class. In my spare time, I like to play the flute and Guzheng. I used to teach my brother playing Guzheng at weekends. In the third International Chinese Arts Festival Western Orchestral Music Contest, I won the Silver Award for playing the flute in the Senior Group, and in 2012, I got the Third Prize for Chinese Zither Performance of Junior Group of Chinese National Instruments International Competition in the fourth International Chinese Arts Festival. Learning musical instruments has exercised my perseverance, as I need a lot of time to practice. At the same time, I studied music theory and Art history. These all broaden my horizons and inform me of the diversity of culture. I think practice is the best way to learn, and therefore I like travelling. Travelling gives me the opportunity to experience different cultures in-person, and meet people from across the world. I also enjoy volunteering. Last year I joined the Lion Clubs International in Hong Kong; one of the activities I undertook was visiting disadvantaged children and teaching them to do handwork. I was moved by their pureness and thirst for knowledge. Another activity was preparing lunch for the elderly. This task required a delegation and a clear division of work to make our work most efficient. These experiences are very valuable, enriching my life and making it meaningful. I hope to continue to volunteer whilst at university. After graduation, I dream to become an English teacher and design courses for students to help them learn English and Chinese in the most efficient way. I believe that by combining the traditional Chinese and Western education modes, my students will acquire a comprehensive understanding of the subject. Studying in the UK will help me towards my career goals. 45 (example of an international application) Did you know...  Students can major in History, Literature, Art History, Philosophy, Politics, Media Studies or Sociology.  And take optional modules across literature, film, philosophy, history of art, history, linguistics, politics, sociology and modern languages.  Students are employed in a variety of careers in the media, journalism, publishing, local government, voluntary agencies, librarianship, finance, management and other fields.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>BSC B473 LIBERAL ARTS</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LIBERAL ARTS</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
         <v>27</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>LIBERAL ARTS</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>(example of an international application) My first contact with English literature was at my high school. My English teacher showed us part of the movie Pride and Prejudice; I could not wait to watch the whole movie when I went home! After watching the movie several times, I tried to read the original book. At the time, I found the book difficult to understand, however the elegance and humour of the literature fascinated me deeply, and inspired me to find out more. I am looking forward to progressing my English ability and appreciating more excellent literary works in their original versions in the university. I enjoy reading masterpieces and watching classical movies. My huge interest in English is also influenced by my mother, who used to be a teacher and later founded a tutorial workshop teaching children English lessons. I therefore grew up amongst a group of children younger than me, who I would teach and support. Although it is hard work to teach others, I found that it was me who benefited most during the process. By helping these children, I would gain a deeper understanding and knowledge of the topic. Teaching has also enabled me to develop my communication skills and I feel satisfied helping others, whilst improving myself. With the support from my mother, I spent several months designing an English course to help children in China learn English; the course consists of 20 parts, including learning of the alphabet, grammar, and the practical application of language. Gradually, I found that my knowledge of English is not enough at all, just the tip of the iceberg, and I am passionate about finding out more. Through this process not only did I learn more English literature knowledge, but also fell in love with European culture and history. I got fine results in my courses including History, Geography and Politics, and ranked Top 5 in my class. In my spare time, I like to play the flute and Guzheng. I used to teach my brother playing Guzheng at weekends. In the third International Chinese Arts Festival Western Orchestral Music Contest, I won the Silver Award for playing the flute in the Senior Group, and in 2012, I got the Third Prize for Chinese Zither Performance of Junior Group of Chinese National Instruments International Competition in the fourth International Chinese Arts Festival. Learning musical instruments has exercised my perseverance, as I need a lot of time to practice. At the same time, I studied music theory and Art history. These all broaden my horizons and inform me of the diversity of culture. I think practice is the best way to learn, and therefore I like travelling. Travelling gives me the opportunity to experience different cultures in-person, and meet people from across the world. I also enjoy volunteering. Last year I joined the Lion Clubs International in Hong Kong; one of the activities I undertook was visiting disadvantaged children and teaching them to do handwork. I was moved by their pureness and thirst for knowledge. Another activity was preparing lunch for the elderly. This task required a delegation and a clear division of work to make our work most efficient. These experiences are very valuable, enriching my life and making it meaningful. I hope to continue to volunteer whilst at university. After graduation, I dream to become an English teacher and design courses for students to help them learn English and Chinese in the most efficient way. I believe that by combining the traditional Chinese and Western education modes, my students will acquire a comprehensive understanding of the subject. Studying in the UK will help me towards my career goals. 45 (example of an international application) Did you know...  Students can major in History, Literature, Art History, Philosophy, Politics, Media Studies or Sociology.  And take optional modules across literature, film, philosophy, history of art, history, linguistics, politics, sociology and modern languages.  Students are employed in a variety of careers in the media, journalism, publishing, local government, voluntary agencies, librarianship, finance, management and other fields.</t>
-        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
+        <v>1027</v>
+      </c>
+      <c r="B29" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>(example of an BTEC application) Engineering is the future; new technologies around the world are exciting and varied, and I would relish the chance of specialising in design engineer work coupled with robotic engineering. Having enjoyed an inspirational relationship with my grandfather, who was a sonar/acoustics engineer with patented designs in the nuclear marine department of the Military of Defence, I have always been encouraged to look for answers using my love of physics and maths. At a young age, I enjoyed taking damaged toys apart and trying to fix them. Very quickly I learnt how to wire a simple motor and battery circuit. After that I learnt how to solder, and design on 2D and 3D software on computers. I now design and print on my own 3D printer, proudly purchased by me, and pushing my software limits to achieve new and improved ideas. I have designed my own electric claw machine for my GCSE DT project. I am now designing my own remote controlled robotic arm for my college engineering project. This has been inspired by the work carried out at Headley Court and the rehabilitation of the amputees and the work carried out at Boston Dynamics with their advanced robotic dexterity. On a personal side, I have worked part-time for the last two years at an extremely popular beach cafe. Progressing from washing up (essential training for any 14-year-old!), to waiting tables and now a student chef. I train the new, young staff and organise their time management which can be quite challenging. I also enjoy racket sports and have represented my county in squash. I am also a qualified young leader with our Scout group. I believe the experience of juggling a busy part-time job alongside studying for my GCSEs, BTEC, commitments to the Scout troop and maintaining my sports interests have taught me how to manage my time and focus. I appreciate timelines and deadlines. I understand and respect management decisions. I enjoy working within a team, be it at work or at college, like problem solving and I enjoy the social side of team building, plus I have a good sense of humour. I am really looking forward to going to university to expand my knowledge and love of this subject and to be with people who appreciate how exciting and important engineering is and will be for the future.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>BSC H439 ROBOTIC ENGINEERING</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ROBOTIC ENGINEERING</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
         <v>28</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>ROBOTIC ENGINEERING</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>(example of an BTEC application) Engineering is the future; new technologies around the world are exciting and varied, and I would relish the chance of specialising in design engineer work coupled with robotic engineering. Having enjoyed an inspirational relationship with my grandfather, who was a sonar/acoustics engineer with patented designs in the nuclear marine department of the Military of Defence, I have always been encouraged to look for answers using my love of physics and maths. At a young age, I enjoyed taking damaged toys apart and trying to fix them. Very quickly I learnt how to wire a simple motor and battery circuit. After that I learnt how to solder, and design on 2D and 3D software on computers. I now design and print on my own 3D printer, proudly purchased by me, and pushing my software limits to achieve new and improved ideas. I have designed my own electric claw machine for my GCSE DT project. I am now designing my own remote controlled robotic arm for my college engineering project. This has been inspired by the work carried out at Headley Court and the rehabilitation of the amputees and the work carried out at Boston Dynamics with their advanced robotic dexterity. On a personal side, I have worked part-time for the last two years at an extremely popular beach cafe. Progressing from washing up (essential training for any 14-year-old!), to waiting tables and now a student chef. I train the new, young staff and organise their time management which can be quite challenging. I also enjoy racket sports and have represented my county in squash. I am also a qualified young leader with our Scout group. I believe the experience of juggling a busy part-time job alongside studying for my GCSEs, BTEC, commitments to the Scout troop and maintaining my sports interests have taught me how to manage my time and focus. I appreciate timelines and deadlines. I understand and respect management decisions. I enjoy working within a team, be it at work or at college, like problem solving and I enjoy the social side of team building, plus I have a good sense of humour. I am really looking forward to going to university to expand my knowledge and love of this subject and to be with people who appreciate how exciting and important engineering is and will be for the future.</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>